<commit_message>
Contenção rápida: rótulos do diagrama da laje com carga na placa (kN/m) igual à tabela, além da pressão (kN/m²)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01STLw65tKW2EfXfQSwTwwMc
</commit_message>
<xml_diff>
--- a/3 - EMPUXO DE MUROS DE ARRIMO.xlsx
+++ b/3 - EMPUXO DE MUROS DE ARRIMO.xlsx
@@ -3723,7 +3723,7 @@
               <a:rPr lang="pt-BR" sz="1100" b="1">
                 <a:latin typeface="Aptos Narrow"/>
               </a:rPr>
-              <a:t>LAJE ALVEOLAR – PRESSÃO NOS PAINÉIS (kN/m²)</a:t>
+              <a:t>LAJE ALVEOLAR – PRESSÃO (kN/m²) E CARGA NA PLACA (kN/m)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -4614,7 +4614,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>σ,topo = 2,64 kN/m²</c:v>
+                  <c:v>σq = 2,64 kN/m² (Sc)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -4686,7 +4686,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>σ,base = 26,39 kN/m²</c:v>
+                  <c:v>σ,base = 26,39 kN/m² = solo 23,75 + Sc 2,64</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -4758,7 +4758,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>P1: 26,4</c:v>
+                  <c:v>P1: g = 29,69 | q = 3,30 kN/m</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -4830,7 +4830,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>P2: 14,5</c:v>
+                  <c:v>P2: g = 14,85 | q = 3,30 kN/m</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -14986,10 +14986,10 @@
       <c r="S106" s="221"/>
       <c r="T106" s="221"/>
     </row>
-    <row r="108" ht="45" customHeight="1">
+    <row r="108" ht="75" customHeight="1">
       <c r="K108" s="220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gráficos de dispersão desenhados a partir da tabela de coordenadas do item 6.1. À esquerda: pilar com a carga trapezoidal (kN/m), a resultante E e as reações. À direita: parede de placas alveolares com a pressão real (vermelho) e a pressão adotada em cada painel (azul, constante = valor da borda inferior).</t>
+          <t xml:space="preserve">Gráficos de dispersão desenhados a partir da tabela de coordenadas do item 6.1. À esquerda: pilar com a carga trapezoidal (kN/m), a resultante E e as reações. À direita: parede de placas alveolares com a pressão real (vermelho) e a pressão adotada em cada painel (azul, constante = valor da borda inferior). O eixo está em PRESSÃO (kN/m²); os rótulos P1, P2… trazem a CARGA NA PLACA (kN/m) = pressão × bw, a mesma da tabela 5.2 (ex.: 23,75 × 1,25 = 29,69 kN/m de solo e 2,64 × 1,25 = 3,30 kN/m de sobrecarga).</t>
         </is>
       </c>
       <c r="L108" s="220"/>
@@ -15875,7 +15875,7 @@
     </row>
     <row r="222">
       <c r="K222" s="237">
-        <f>"σ,topo = "&amp;FIXED($L$47,2)&amp;" kN/m²"</f>
+        <f>"σq = "&amp;FIXED($L$47,2)&amp;" kN/m² (Sc)"</f>
       </c>
       <c r="L222" s="227">
         <f>$L$47</f>
@@ -15886,7 +15886,7 @@
     </row>
     <row r="223">
       <c r="K223" s="237">
-        <f>"σ,base = "&amp;FIXED($L$48,2)&amp;" kN/m²"</f>
+        <f>"σ,base = "&amp;FIXED($L$48,2)&amp;" kN/m² = solo "&amp;FIXED($L$49,2)&amp;" + Sc "&amp;FIXED($L$47,2)</f>
       </c>
       <c r="L223" s="227">
         <f>$L$48</f>
@@ -15897,7 +15897,7 @@
     </row>
     <row r="224">
       <c r="K224" s="237">
-        <f>IF(L95="","","P1: "&amp;FIXED(P95,1))</f>
+        <f>IF(L95="","","P1: g = "&amp;FIXED(Q95,2)&amp;" | q = "&amp;FIXED(R95,2)&amp;" kN/m")</f>
       </c>
       <c r="L224" s="227">
         <f>IF(L95="",NA(),P95)</f>
@@ -15908,7 +15908,7 @@
     </row>
     <row r="225">
       <c r="K225" s="237">
-        <f>IF(L96="","","P2: "&amp;FIXED(P96,1))</f>
+        <f>IF(L96="","","P2: g = "&amp;FIXED(Q96,2)&amp;" | q = "&amp;FIXED(R96,2)&amp;" kN/m")</f>
       </c>
       <c r="L225" s="227">
         <f>IF(L96="",NA(),P96)</f>
@@ -15919,7 +15919,7 @@
     </row>
     <row r="226">
       <c r="K226" s="237">
-        <f>IF(L97="","","P3: "&amp;FIXED(P97,1))</f>
+        <f>IF(L97="","","P3: g = "&amp;FIXED(Q97,2)&amp;" | q = "&amp;FIXED(R97,2)&amp;" kN/m")</f>
       </c>
       <c r="L226" s="227">
         <f>IF(L97="",NA(),P97)</f>
@@ -15930,7 +15930,7 @@
     </row>
     <row r="227">
       <c r="K227" s="237">
-        <f>IF(L98="","","P4: "&amp;FIXED(P98,1))</f>
+        <f>IF(L98="","","P4: g = "&amp;FIXED(Q98,2)&amp;" | q = "&amp;FIXED(R98,2)&amp;" kN/m")</f>
       </c>
       <c r="L227" s="227">
         <f>IF(L98="",NA(),P98)</f>
@@ -15941,7 +15941,7 @@
     </row>
     <row r="228">
       <c r="K228" s="237">
-        <f>IF(L99="","","P5: "&amp;FIXED(P99,1))</f>
+        <f>IF(L99="","","P5: g = "&amp;FIXED(Q99,2)&amp;" | q = "&amp;FIXED(R99,2)&amp;" kN/m")</f>
       </c>
       <c r="L228" s="227">
         <f>IF(L99="",NA(),P99)</f>
@@ -15952,7 +15952,7 @@
     </row>
     <row r="229">
       <c r="K229" s="237">
-        <f>IF(L100="","","P6: "&amp;FIXED(P100,1))</f>
+        <f>IF(L100="","","P6: g = "&amp;FIXED(Q100,2)&amp;" | q = "&amp;FIXED(R100,2)&amp;" kN/m")</f>
       </c>
       <c r="L229" s="227">
         <f>IF(L100="",NA(),P100)</f>
@@ -15963,7 +15963,7 @@
     </row>
     <row r="230">
       <c r="K230" s="237">
-        <f>IF(L101="","","P7: "&amp;FIXED(P101,1))</f>
+        <f>IF(L101="","","P7: g = "&amp;FIXED(Q101,2)&amp;" | q = "&amp;FIXED(R101,2)&amp;" kN/m")</f>
       </c>
       <c r="L230" s="227">
         <f>IF(L101="",NA(),P101)</f>
@@ -15974,7 +15974,7 @@
     </row>
     <row r="231">
       <c r="K231" s="237">
-        <f>IF(L102="","","P8: "&amp;FIXED(P102,1))</f>
+        <f>IF(L102="","","P8: g = "&amp;FIXED(Q102,2)&amp;" | q = "&amp;FIXED(R102,2)&amp;" kN/m")</f>
       </c>
       <c r="L231" s="227">
         <f>IF(L102="",NA(),P102)</f>
@@ -15985,7 +15985,7 @@
     </row>
     <row r="232">
       <c r="K232" s="237">
-        <f>IF(L103="","","P9: "&amp;FIXED(P103,1))</f>
+        <f>IF(L103="","","P9: g = "&amp;FIXED(Q103,2)&amp;" | q = "&amp;FIXED(R103,2)&amp;" kN/m")</f>
       </c>
       <c r="L232" s="227">
         <f>IF(L103="",NA(),P103)</f>
@@ -15996,7 +15996,7 @@
     </row>
     <row r="233">
       <c r="K233" s="237">
-        <f>IF(L104="","","P10: "&amp;FIXED(P104,1))</f>
+        <f>IF(L104="","","P10: g = "&amp;FIXED(Q104,2)&amp;" | q = "&amp;FIXED(R104,2)&amp;" kN/m")</f>
       </c>
       <c r="L233" s="227">
         <f>IF(L104="",NA(),P104)</f>

</xml_diff>

<commit_message>
Aba DIMENSIONAMENTO PILAR: pilar como viga (flexão simples no vão e na base), armadura simétrica e estribos pelo Modelo I
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01STLw65tKW2EfXfQSwTwwMc
</commit_message>
<xml_diff>
--- a/3 - EMPUXO DE MUROS DE ARRIMO.xlsx
+++ b/3 - EMPUXO DE MUROS DE ARRIMO.xlsx
@@ -14,6 +14,7 @@
   </bookViews>
   <sheets>
     <sheet name="CONTENÇÃO RÁPIDA" sheetId="11" r:id="rId99"/>
+    <sheet name="DIMENSIONAMENTO PILAR" sheetId="12" r:id="rId98"/>
     <sheet name="MURO DE ARRIMO" sheetId="1" r:id="rId1"/>
     <sheet name="DADOS DO SOLO" sheetId="6" r:id="rId2"/>
     <sheet name="ASSENTAMENTO" sheetId="4" r:id="rId3"/>
@@ -24,6 +25,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'CONTENÇÃO RÁPIDA'!$K$1:$T$259</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'DIMENSIONAMENTO PILAR'!$K$1:$T$127</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1" iterateCount="1000"/>
   <extLst>
@@ -16527,4 +16529,2012 @@
   <pageSetup paperSize="9" fitToHeight="0" orientation="portrait"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="K1:T127"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="10" max="10" width="2.7109375" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="9.7109375" customWidth="1"/>
+    <col min="14" max="14" width="27.7109375" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="K1" s="219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIMENSIONAMENTO DO PILAR COMO VIGA BIAPOIADA – FLEXÃO SIMPLES E ESTRIBOS (NBR 6118)</t>
+        </is>
+      </c>
+      <c r="L1" s="219"/>
+      <c r="M1" s="219"/>
+      <c r="N1" s="219"/>
+      <c r="O1" s="219"/>
+      <c r="P1" s="219"/>
+      <c r="Q1" s="219"/>
+      <c r="R1" s="219"/>
+      <c r="S1" s="219"/>
+      <c r="T1" s="219"/>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="K2" s="239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARMADURA LONGITUDINAL</t>
+        </is>
+      </c>
+      <c r="L2" s="239"/>
+      <c r="M2" s="240">
+        <f>$L$100&amp;" Ø"&amp;$L$42&amp;" em cada face (simétrica)"</f>
+      </c>
+      <c r="N2" s="240"/>
+      <c r="O2" s="240">
+        <f>"As,ef = "&amp;FIXED($L$101,2)&amp;" cm²/face | total "&amp;FIXED($L$102,2)&amp;" cm²"</f>
+      </c>
+      <c r="P2" s="240"/>
+      <c r="Q2" s="240"/>
+      <c r="R2" s="240">
+        <f>"ρ = "&amp;FIXED($L$103,2)&amp;" % | "&amp;IF($L$105&lt;$L$104,"NÃO CABE","cabe na face")</f>
+      </c>
+      <c r="S2" s="240"/>
+      <c r="T2" s="240"/>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="K3" s="239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESTRIBOS</t>
+        </is>
+      </c>
+      <c r="L3" s="239"/>
+      <c r="M3" s="240">
+        <f>"Ø"&amp;$L$41&amp;" c/"&amp;$L$125&amp;" ("&amp;$L$43&amp;" ramos)"</f>
+      </c>
+      <c r="N3" s="240"/>
+      <c r="O3" s="240">
+        <f>"Asw = "&amp;FIXED($L$121,2)&amp;" cm²/m"</f>
+      </c>
+      <c r="P3" s="240"/>
+      <c r="Q3" s="240"/>
+      <c r="R3" s="240">
+        <f>"Vsd = "&amp;FIXED($L$111,1)&amp;" kN | VRd2 = "&amp;FIXED($L$112,1)&amp;" kN"</f>
+      </c>
+      <c r="S3" s="240"/>
+      <c r="T3" s="240"/>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="K4" s="239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESFORÇOS DE CÁLCULO</t>
+        </is>
+      </c>
+      <c r="L4" s="239"/>
+      <c r="M4" s="240">
+        <f>"Md+ = "&amp;FIXED($L$72,2)&amp;" | Md− = "&amp;FIXED($L$83,2)&amp;" kN·m"</f>
+      </c>
+      <c r="N4" s="240"/>
+      <c r="O4" s="240">
+        <f>"Md,lim = "&amp;FIXED($L$67,2)&amp;" kN·m"</f>
+      </c>
+      <c r="P4" s="240"/>
+      <c r="Q4" s="240"/>
+      <c r="R4" s="240">
+        <f>"Modelo: "&amp;$L$45&amp;" | seção "&amp;$L$39&amp;"×"&amp;$L$38</f>
+      </c>
+      <c r="S4" s="240"/>
+      <c r="T4" s="240"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="K6" s="220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Como usar: células CINZA são entradas; os esforços vêm da aba CONTENÇÃO RÁPIDA (pode sobrescrever). Pilar tratado como viga (flexão simples, sem a força normal). Armadura longitudinal SIMÉTRICA: as duas faces recebem a mesma armadura, dimensionada pela pior situação entre a seção do vão (M+) e a da base (M−). Estribos pelo Modelo I (θ = 45°, α = 90°).</t>
+        </is>
+      </c>
+      <c r="L6" s="220"/>
+      <c r="M6" s="220"/>
+      <c r="N6" s="220"/>
+      <c r="O6" s="220"/>
+      <c r="P6" s="220"/>
+      <c r="Q6" s="220"/>
+      <c r="R6" s="220"/>
+      <c r="S6" s="220"/>
+      <c r="T6" s="220"/>
+    </row>
+    <row r="8">
+      <c r="K8" s="221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESUMO DAS VERIFICAÇÕES E ARMADURAS</t>
+        </is>
+      </c>
+      <c r="L8" s="221"/>
+      <c r="M8" s="221"/>
+      <c r="N8" s="221"/>
+      <c r="O8" s="221"/>
+      <c r="P8" s="221"/>
+      <c r="Q8" s="221"/>
+      <c r="R8" s="221"/>
+      <c r="S8" s="221"/>
+      <c r="T8" s="221"/>
+    </row>
+    <row r="10">
+      <c r="K10" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Item</t>
+        </is>
+      </c>
+      <c r="L10" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resultado</t>
+        </is>
+      </c>
+      <c r="M10" s="235"/>
+      <c r="N10" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status</t>
+        </is>
+      </c>
+      <c r="O10" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O que é</t>
+        </is>
+      </c>
+      <c r="P10" s="235"/>
+      <c r="Q10" s="235"/>
+      <c r="R10" s="235"/>
+      <c r="S10" s="235"/>
+      <c r="T10" s="235"/>
+    </row>
+    <row r="11">
+      <c r="K11" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Esforços</t>
+        </is>
+      </c>
+      <c r="L11" s="236">
+        <f>"Md+ = "&amp;FIXED($L$72,1)&amp;" | Md− = "&amp;FIXED($L$83,1)</f>
+      </c>
+      <c r="M11" s="236"/>
+      <c r="N11" s="232">
+        <f>IF(ISNA(MATCH($L$45,'CONTENÇÃO RÁPIDA'!$K$74:$K$76,0)),"Rever: modelo inválido","Ok")</f>
+      </c>
+      <c r="O11" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Momentos de cálculo (kN·m) do modelo escolhido – item 1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="K12" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aviso</t>
+        </is>
+      </c>
+      <c r="L12" s="234">
+        <f>IF(MAX($L$72,$L$83)&gt;$L$67,"⚠ Armadura dupla: a seção "&amp;$L$39&amp;"×"&amp;$L$38&amp;" é pequena para Md = "&amp;FIXED(MAX($L$72,$L$83),1)&amp;" kN·m. Para armadura simples use h ≥ "&amp;ROUNDUP($L$68+$L$64,0)&amp;" cm.","Flexão simples (sem a força normal): se o pilar tiver compressão relevante, confira a flexo-compressão no programa.")</f>
+      </c>
+      <c r="M12" s="234"/>
+      <c r="N12" s="234"/>
+      <c r="O12" s="234"/>
+      <c r="P12" s="234"/>
+      <c r="Q12" s="234"/>
+      <c r="R12" s="234"/>
+      <c r="S12" s="234"/>
+      <c r="T12" s="234"/>
+    </row>
+    <row r="13">
+      <c r="K13" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seção do vão</t>
+        </is>
+      </c>
+      <c r="L13" s="236">
+        <f>$L$73</f>
+      </c>
+      <c r="M13" s="236"/>
+      <c r="N13" s="232">
+        <f>IF($L$72=0,"Não se aplica (M = 0)",IF($L$72&lt;=$L$67,"Ok","Arm. dupla – ver d,mín"))</f>
+      </c>
+      <c r="O13" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flexão com M+ – item 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="K14" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seção da base</t>
+        </is>
+      </c>
+      <c r="L14" s="236">
+        <f>$L$84</f>
+      </c>
+      <c r="M14" s="236"/>
+      <c r="N14" s="232">
+        <f>IF($L$83=0,"Não se aplica (M = 0)",IF($L$83&lt;=$L$67,"Ok","Arm. dupla – ver d,mín"))</f>
+      </c>
+      <c r="O14" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flexão com M− – item 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="K15" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Arm. por face</t>
+        </is>
+      </c>
+      <c r="L15" s="236">
+        <f>$L$100&amp;" Ø"&amp;$L$42&amp;" ("&amp;FIXED($L$101,2)&amp;" cm²)"</f>
+      </c>
+      <c r="M15" s="236"/>
+      <c r="N15" s="232">
+        <f>IF($L$105&lt;$L$104,"Não cabe: aumentar b ou Ø,l","Ok")</f>
+      </c>
+      <c r="O15" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mesma armadura nas duas faces (simétrica) – item 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="K16" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Taxa total</t>
+        </is>
+      </c>
+      <c r="L16" s="236">
+        <f>FIXED($L$103,2)&amp;" %"</f>
+      </c>
+      <c r="M16" s="236"/>
+      <c r="N16" s="232">
+        <f>IF($L$103&gt;4,"Rever: taxa &gt; 4%",IF($L$103&lt;0.4,"Rever: taxa &lt; 0,4%","Ok"))</f>
+      </c>
+      <c r="O16" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura total / Ac – item 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="K17" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Biela</t>
+        </is>
+      </c>
+      <c r="L17" s="236">
+        <f>FIXED($L$111,1)&amp;" ≤ "&amp;FIXED($L$112,1)&amp;" kN"</f>
+      </c>
+      <c r="M17" s="236"/>
+      <c r="N17" s="232">
+        <f>IF($L$111&lt;=$L$112,"Ok","Aumentar seção ou fck")</f>
+      </c>
+      <c r="O17" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vsd ≤ VRd2 – item 6.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="K18" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estribos</t>
+        </is>
+      </c>
+      <c r="L18" s="236">
+        <f>"Ø"&amp;$L$41&amp;" c/"&amp;$L$125&amp;" ("&amp;$L$43&amp;" ramos)"</f>
+      </c>
+      <c r="M18" s="236"/>
+      <c r="N18" s="232">
+        <f>IF($L$125&lt;5,"s &lt; 5 cm – aumentar Ø,t",IF($L$126&gt;=$L$121,"Ok","Rever"))</f>
+      </c>
+      <c r="O18" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estribos em toda a altura do pilar – item 6.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="K26" s="221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 . DADOS DE ENTRADA</t>
+        </is>
+      </c>
+      <c r="L26" s="221"/>
+      <c r="M26" s="221"/>
+      <c r="N26" s="221"/>
+      <c r="O26" s="221"/>
+      <c r="P26" s="221"/>
+      <c r="Q26" s="221"/>
+      <c r="R26" s="221"/>
+      <c r="S26" s="221"/>
+      <c r="T26" s="221"/>
+    </row>
+    <row r="28">
+      <c r="K28" s="222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.1 Coeficientes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="K29" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">γf</t>
+        </is>
+      </c>
+      <c r="L29" s="224">
+        <v>1.4</v>
+      </c>
+      <c r="M29" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O29" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coeficiente de majoração das cargas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="K30" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">γc</t>
+        </is>
+      </c>
+      <c r="L30" s="224">
+        <v>1.4</v>
+      </c>
+      <c r="M30" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O30" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coeficiente de minoração do concreto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="K31" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">γs</t>
+        </is>
+      </c>
+      <c r="L31" s="224">
+        <v>1.15</v>
+      </c>
+      <c r="M31" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O31" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coeficiente de minoração do aço.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="K32" s="222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.2 Materiais</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="K33" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fck</t>
+        </is>
+      </c>
+      <c r="L33" s="224">
+        <v>30</v>
+      </c>
+      <c r="M33" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPa</t>
+        </is>
+      </c>
+      <c r="N33" s="232">
+        <f>IF(OR($L$33&lt;20,$L$33&gt;50),"Rever: fck entre 20 e 50 MPa","Ok")</f>
+      </c>
+      <c r="O33" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistência característica do concreto (até 50 MPa).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="K34" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fyk</t>
+        </is>
+      </c>
+      <c r="L34" s="224">
+        <v>500</v>
+      </c>
+      <c r="M34" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPa</t>
+        </is>
+      </c>
+      <c r="O34" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aço da armadura longitudinal (CA-50).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="K35" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fywk</t>
+        </is>
+      </c>
+      <c r="L35" s="224">
+        <v>500</v>
+      </c>
+      <c r="M35" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPa</t>
+        </is>
+      </c>
+      <c r="O35" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aço dos estribos (CA-50 = 500; CA-60 = 600).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="K36" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d,máx</t>
+        </is>
+      </c>
+      <c r="L36" s="224">
+        <v>19</v>
+      </c>
+      <c r="M36" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="O36" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diâmetro máximo do agregado (brita 1 = 19 mm).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="K37" s="222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.3 Seção do pilar</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="K38" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">h</t>
+        </is>
+      </c>
+      <c r="L38" s="224">
+        <v>30</v>
+      </c>
+      <c r="M38" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O38" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dimensão na direção do empuxo (altura da seção que resiste à flexão).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="K39" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b</t>
+        </is>
+      </c>
+      <c r="L39" s="224">
+        <v>20</v>
+      </c>
+      <c r="M39" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O39" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dimensão da face onde ficam as barras (largura da 'viga').</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="K40" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c</t>
+        </is>
+      </c>
+      <c r="L40" s="224">
+        <v>3</v>
+      </c>
+      <c r="M40" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O40" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cobrimento (CAA II: pilar 3,0 cm).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="K41" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ø,t</t>
+        </is>
+      </c>
+      <c r="L41" s="224">
+        <v>6.3</v>
+      </c>
+      <c r="M41" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="O41" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bitola do estribo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="K42" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ø,l</t>
+        </is>
+      </c>
+      <c r="L42" s="224">
+        <v>12.5</v>
+      </c>
+      <c r="M42" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="N42" s="232">
+        <f>IF($L$42&lt;10,"Rever: pilar pede Ø ≥ 10 mm",IF($L$42&gt;$L$39*10/8,"Rever: Ø &gt; b/8","Ok"))</f>
+      </c>
+      <c r="O42" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bitola da armadura longitudinal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="K43" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ramos</t>
+        </is>
+      </c>
+      <c r="L43" s="224">
+        <v>2</v>
+      </c>
+      <c r="M43" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O43" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ramos de cada estribo (estribo fechado = 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="K44" s="222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.4 Esforços característicos (da aba CONTENÇÃO RÁPIDA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="K45" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Modelo</t>
+        </is>
+      </c>
+      <c r="L45" s="224" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Biapoiado</t>
+        </is>
+      </c>
+      <c r="M45" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N45" s="232">
+        <f>IF(ISNA(MATCH($L$45,'CONTENÇÃO RÁPIDA'!$K$74:$K$76,0)),"Rever: modelo inválido","Ok")</f>
+      </c>
+      <c r="O45" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Modelo do pilar: Biapoiado (padrão), Engaste-apoio ou Balanço.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="K46" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mk+</t>
+        </is>
+      </c>
+      <c r="L46" s="225">
+        <f>MAX(0,IFERROR(INDEX('CONTENÇÃO RÁPIDA'!$O$74:$O$76,MATCH($L$45,'CONTENÇÃO RÁPIDA'!$K$74:$K$76,0)),0))</f>
+      </c>
+      <c r="M46" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kN·m</t>
+        </is>
+      </c>
+      <c r="O46" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Momento positivo máximo (vão) – tração na face externa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="K47" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mk−</t>
+        </is>
+      </c>
+      <c r="L47" s="225">
+        <f>ABS(MIN(0,IFERROR(INDEX('CONTENÇÃO RÁPIDA'!$N$74:$N$76,MATCH($L$45,'CONTENÇÃO RÁPIDA'!$K$74:$K$76,0)),0)))</f>
+      </c>
+      <c r="M47" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kN·m</t>
+        </is>
+      </c>
+      <c r="O47" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Momento negativo na base (em módulo) – tração na face do solo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="K48" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vk</t>
+        </is>
+      </c>
+      <c r="L48" s="225">
+        <f>MAX(IFERROR(INDEX('CONTENÇÃO RÁPIDA'!$L$74:$L$76,MATCH($L$45,'CONTENÇÃO RÁPIDA'!$K$74:$K$76,0)),0),IFERROR(INDEX('CONTENÇÃO RÁPIDA'!$M$74:$M$76,MATCH($L$45,'CONTENÇÃO RÁPIDA'!$K$74:$K$76,0)),0))</f>
+      </c>
+      <c r="M48" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kN</t>
+        </is>
+      </c>
+      <c r="O48" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maior cortante = maior reação (R,topo ou R,base).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="K49" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nk</t>
+        </is>
+      </c>
+      <c r="L49" s="224">
+        <v>0</v>
+      </c>
+      <c r="M49" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kN</t>
+        </is>
+      </c>
+      <c r="O49" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Força normal no pilar (compressão). Usada só na armadura mínima de pilar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="K50" s="222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.5 Tabela ρ,mín (NBR 6118, tab. 17.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="K51" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fck (MPa)</t>
+        </is>
+      </c>
+      <c r="L51" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ρ,mín (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="K52" s="237">
+        <v>20</v>
+      </c>
+      <c r="L52" s="226">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="K53" s="237">
+        <v>25</v>
+      </c>
+      <c r="L53" s="226">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="K54" s="237">
+        <v>30</v>
+      </c>
+      <c r="L54" s="226">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="K55" s="237">
+        <v>35</v>
+      </c>
+      <c r="L55" s="226">
+        <v>0.164</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="K56" s="237">
+        <v>40</v>
+      </c>
+      <c r="L56" s="226">
+        <v>0.179</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="K57" s="237">
+        <v>45</v>
+      </c>
+      <c r="L57" s="226">
+        <v>0.194</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="K58" s="237">
+        <v>50</v>
+      </c>
+      <c r="L58" s="226">
+        <v>0.208</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="K60" s="221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 . PARÂMETROS DE CÁLCULO</t>
+        </is>
+      </c>
+      <c r="L60" s="221"/>
+      <c r="M60" s="221"/>
+      <c r="N60" s="221"/>
+      <c r="O60" s="221"/>
+      <c r="P60" s="221"/>
+      <c r="Q60" s="221"/>
+      <c r="R60" s="221"/>
+      <c r="S60" s="221"/>
+      <c r="T60" s="221"/>
+    </row>
+    <row r="62">
+      <c r="K62" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fcd</t>
+        </is>
+      </c>
+      <c r="L62" s="227">
+        <f>$L$33/$L$30</f>
+      </c>
+      <c r="M62" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPa</t>
+        </is>
+      </c>
+      <c r="O62" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistência de cálculo do concreto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="K63" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fyd</t>
+        </is>
+      </c>
+      <c r="L63" s="227">
+        <f>$L$34/$L$31</f>
+      </c>
+      <c r="M63" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPa</t>
+        </is>
+      </c>
+      <c r="O63" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistência de cálculo do aço.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="K64" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d'</t>
+        </is>
+      </c>
+      <c r="L64" s="227">
+        <f>$L$40+$L$41/10+$L$42/20</f>
+      </c>
+      <c r="M64" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O64" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Distância da face ao eixo das barras (c + Ø,t + Ø,l/2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="K65" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d</t>
+        </is>
+      </c>
+      <c r="L65" s="227">
+        <f>$L$38-$L$64</f>
+      </c>
+      <c r="M65" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O65" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Altura útil (h − d').</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="K66" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(x/d)lim</t>
+        </is>
+      </c>
+      <c r="L66" s="227">
+        <v>0.45</v>
+      </c>
+      <c r="M66" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O66" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limite da linha neutra para fck ≤ 50 MPa (ductilidade).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="K67" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Md,lim</t>
+        </is>
+      </c>
+      <c r="L67" s="227">
+        <f>0.68*$L$39*$L$65^2*$L$62/10*$L$66*(1-0.4*$L$66)/100</f>
+      </c>
+      <c r="M67" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kN·m</t>
+        </is>
+      </c>
+      <c r="O67" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maior momento de cálculo só com armadura simples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="K68" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d,mín</t>
+        </is>
+      </c>
+      <c r="L68" s="227">
+        <f>SQRT(MAX($L$46,$L$47)*$L$29*100/(0.68*$L$39*$L$62/10*$L$66*(1-0.4*$L$66)))</f>
+      </c>
+      <c r="M68" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="N68" s="232">
+        <f>IF($L$65&gt;=$L$68,"Ok","Aumentar h para "&amp;ROUNDUP($L$68+$L$64,0)&amp;" cm (arm. simples)")</f>
+      </c>
+      <c r="O68" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Altura útil mínima para armadura simples com o maior momento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="K70" s="221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 . FLEXÃO – SEÇÃO DO VÃO (M+)</t>
+        </is>
+      </c>
+      <c r="L70" s="221"/>
+      <c r="M70" s="221"/>
+      <c r="N70" s="221"/>
+      <c r="O70" s="221"/>
+      <c r="P70" s="221"/>
+      <c r="Q70" s="221"/>
+      <c r="R70" s="221"/>
+      <c r="S70" s="221"/>
+      <c r="T70" s="221"/>
+    </row>
+    <row r="72">
+      <c r="K72" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Md</t>
+        </is>
+      </c>
+      <c r="L72" s="227">
+        <f>$L$46*$L$29</f>
+      </c>
+      <c r="M72" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kN·m</t>
+        </is>
+      </c>
+      <c r="O72" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Momento de cálculo (γf·Mk).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="K73" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tipo</t>
+        </is>
+      </c>
+      <c r="L73" s="230">
+        <f>IF($L$72=0,"Não se aplica (M = 0)",IF($L$72&lt;=$L$67,"Armadura simples","Armadura dupla"))</f>
+      </c>
+      <c r="M73" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N73" s="232">
+        <f>IF($L$72=0,"Não se aplica (M = 0)",IF($L$72&lt;=$L$67,"Ok","Arm. dupla – ver d,mín (item 2)"))</f>
+      </c>
+      <c r="O73" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simples se Md ≤ Md,lim; dupla se maior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="K74" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x</t>
+        </is>
+      </c>
+      <c r="L74" s="227">
+        <f>IF($L$72&lt;=$L$67,1.25*$L$65*(1-SQRT(MAX(0,1-$L$72*100/(0.425*$L$39*$L$65^2*$L$62/10)))),$L$66*$L$65)</f>
+      </c>
+      <c r="M74" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O74" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Profundidade da linha neutra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="K75" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x/d</t>
+        </is>
+      </c>
+      <c r="L75" s="228">
+        <f>IF($L$65=0,0,$L$74/$L$65)</f>
+      </c>
+      <c r="M75" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O75" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Posição relativa da linha neutra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="K76" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Domínio</t>
+        </is>
+      </c>
+      <c r="L76" s="230">
+        <f>IF($L$72=0,"-",IF($L$75&lt;=0.259,"2","3"))</f>
+      </c>
+      <c r="M76" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O76" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Domínio de deformação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="K77" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">σsc</t>
+        </is>
+      </c>
+      <c r="L77" s="227">
+        <f>MIN($L$63,210000*0.0035*MAX(0,$L$74-$L$64)/MAX($L$74,0.001))</f>
+      </c>
+      <c r="M77" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPa</t>
+        </is>
+      </c>
+      <c r="O77" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tensão na armadura comprimida (Es = 210 GPa, εc = 3,5‰), só na armadura dupla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="K78" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As,t</t>
+        </is>
+      </c>
+      <c r="L78" s="227">
+        <f>IF($L$72&lt;=$L$67,$L$72*100/($L$63/10*($L$65-0.4*$L$74)),$L$67*100/($L$63/10*($L$65-0.4*$L$74))+($L$72-$L$67)*100/($L$63/10*($L$65-$L$64)))</f>
+      </c>
+      <c r="M78" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²</t>
+        </is>
+      </c>
+      <c r="O78" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura tracionada – face externa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="K79" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As,c</t>
+        </is>
+      </c>
+      <c r="L79" s="227">
+        <f>IF($L$72&lt;=$L$67,0,($L$72-$L$67)*100/($L$77/10*($L$65-$L$64)))</f>
+      </c>
+      <c r="M79" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²</t>
+        </is>
+      </c>
+      <c r="O79" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura comprimida – face do solo (0 na armadura simples).</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="K81" s="221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 . FLEXÃO – SEÇÃO DA BASE (M−)</t>
+        </is>
+      </c>
+      <c r="L81" s="221"/>
+      <c r="M81" s="221"/>
+      <c r="N81" s="221"/>
+      <c r="O81" s="221"/>
+      <c r="P81" s="221"/>
+      <c r="Q81" s="221"/>
+      <c r="R81" s="221"/>
+      <c r="S81" s="221"/>
+      <c r="T81" s="221"/>
+    </row>
+    <row r="83">
+      <c r="K83" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Md</t>
+        </is>
+      </c>
+      <c r="L83" s="227">
+        <f>$L$47*$L$29</f>
+      </c>
+      <c r="M83" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kN·m</t>
+        </is>
+      </c>
+      <c r="O83" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Momento de cálculo (γf·Mk).</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="K84" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tipo</t>
+        </is>
+      </c>
+      <c r="L84" s="230">
+        <f>IF($L$83=0,"Não se aplica (M = 0)",IF($L$83&lt;=$L$67,"Armadura simples","Armadura dupla"))</f>
+      </c>
+      <c r="M84" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N84" s="232">
+        <f>IF($L$83=0,"Não se aplica (M = 0)",IF($L$83&lt;=$L$67,"Ok","Arm. dupla – ver d,mín (item 2)"))</f>
+      </c>
+      <c r="O84" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simples se Md ≤ Md,lim; dupla se maior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="K85" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x</t>
+        </is>
+      </c>
+      <c r="L85" s="227">
+        <f>IF($L$83&lt;=$L$67,1.25*$L$65*(1-SQRT(MAX(0,1-$L$83*100/(0.425*$L$39*$L$65^2*$L$62/10)))),$L$66*$L$65)</f>
+      </c>
+      <c r="M85" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O85" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Profundidade da linha neutra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="K86" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x/d</t>
+        </is>
+      </c>
+      <c r="L86" s="228">
+        <f>IF($L$65=0,0,$L$85/$L$65)</f>
+      </c>
+      <c r="M86" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O86" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Posição relativa da linha neutra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="K87" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Domínio</t>
+        </is>
+      </c>
+      <c r="L87" s="230">
+        <f>IF($L$83=0,"-",IF($L$86&lt;=0.259,"2","3"))</f>
+      </c>
+      <c r="M87" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O87" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Domínio de deformação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="K88" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">σsc</t>
+        </is>
+      </c>
+      <c r="L88" s="227">
+        <f>MIN($L$63,210000*0.0035*MAX(0,$L$85-$L$64)/MAX($L$85,0.001))</f>
+      </c>
+      <c r="M88" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPa</t>
+        </is>
+      </c>
+      <c r="O88" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tensão na armadura comprimida (Es = 210 GPa, εc = 3,5‰), só na armadura dupla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="K89" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As,t</t>
+        </is>
+      </c>
+      <c r="L89" s="227">
+        <f>IF($L$83&lt;=$L$67,$L$83*100/($L$63/10*($L$65-0.4*$L$85)),$L$67*100/($L$63/10*($L$65-0.4*$L$85))+($L$83-$L$67)*100/($L$63/10*($L$65-$L$64)))</f>
+      </c>
+      <c r="M89" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²</t>
+        </is>
+      </c>
+      <c r="O89" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura tracionada – face do solo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="K90" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As,c</t>
+        </is>
+      </c>
+      <c r="L90" s="227">
+        <f>IF($L$83&lt;=$L$67,0,($L$83-$L$67)*100/($L$88/10*($L$65-$L$64)))</f>
+      </c>
+      <c r="M90" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²</t>
+        </is>
+      </c>
+      <c r="O90" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura comprimida – face externa (0 na armadura simples).</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="K92" s="221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 . ARMADURA LONGITUDINAL SIMÉTRICA (mesma nas duas faces)</t>
+        </is>
+      </c>
+      <c r="L92" s="221"/>
+      <c r="M92" s="221"/>
+      <c r="N92" s="221"/>
+      <c r="O92" s="221"/>
+      <c r="P92" s="221"/>
+      <c r="Q92" s="221"/>
+      <c r="R92" s="221"/>
+      <c r="S92" s="221"/>
+      <c r="T92" s="221"/>
+    </row>
+    <row r="94" ht="32" customHeight="1">
+      <c r="K94" s="220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cada face recebe a maior entre: tração do vão, tração da base, compressão da armadura dupla, mínima de viga (por face) e metade da mínima de pilar (0,4% Ac no total). As mesmas barras seguem por toda a altura, cobrindo as duas seções.</t>
+        </is>
+      </c>
+      <c r="L94" s="220"/>
+      <c r="M94" s="220"/>
+      <c r="N94" s="220"/>
+      <c r="O94" s="220"/>
+      <c r="P94" s="220"/>
+      <c r="Q94" s="220"/>
+      <c r="R94" s="220"/>
+      <c r="S94" s="220"/>
+      <c r="T94" s="220"/>
+    </row>
+    <row r="95">
+      <c r="K95" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ρ,mín</t>
+        </is>
+      </c>
+      <c r="L95" s="228">
+        <f>VLOOKUP($L$33,$K$52:$L$58,2,TRUE)</f>
+      </c>
+      <c r="M95" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="O95" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Taxa mínima de flexão (tabela 1.5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="K96" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As,mín,v</t>
+        </is>
+      </c>
+      <c r="L96" s="227">
+        <f>$L$95/100*$L$39*$L$38</f>
+      </c>
+      <c r="M96" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²</t>
+        </is>
+      </c>
+      <c r="O96" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mínima de viga, por face tracionada: ρ,mín·b·h.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="K97" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As,mín,p</t>
+        </is>
+      </c>
+      <c r="L97" s="227">
+        <f>MAX(0.15*$L$49*$L$29/($L$63/10),0.004*$L$39*$L$38)</f>
+      </c>
+      <c r="M97" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²</t>
+        </is>
+      </c>
+      <c r="O97" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mínima de pilar, total: máx(0,15·Nd/fyd; 0,4%·Ac).</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="K98" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As,face</t>
+        </is>
+      </c>
+      <c r="L98" s="227">
+        <f>MAX($L$78,$L$79,$L$89,$L$90,$L$96,$L$97/2)</f>
+      </c>
+      <c r="M98" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²</t>
+        </is>
+      </c>
+      <c r="O98" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura necessária em cada face.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="K99" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A,barra</t>
+        </is>
+      </c>
+      <c r="L99" s="228">
+        <f>PI()*($L$42/10)^2/4</f>
+      </c>
+      <c r="M99" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²</t>
+        </is>
+      </c>
+      <c r="O99" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Área de uma barra Ø,l.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="K100" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">n</t>
+        </is>
+      </c>
+      <c r="L100" s="229">
+        <f>MAX(2,ROUNDUP($L$98/$L$99,0))</f>
+      </c>
+      <c r="M100" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">un</t>
+        </is>
+      </c>
+      <c r="O100" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Barras em cada face (mínimo 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="K101" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As,ef</t>
+        </is>
+      </c>
+      <c r="L101" s="227">
+        <f>$L$100*$L$99</f>
+      </c>
+      <c r="M101" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²</t>
+        </is>
+      </c>
+      <c r="O101" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura efetiva em cada face.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="K102" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As,total</t>
+        </is>
+      </c>
+      <c r="L102" s="227">
+        <f>2*$L$101</f>
+      </c>
+      <c r="M102" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²</t>
+        </is>
+      </c>
+      <c r="O102" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura total na seção (duas faces).</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="K103" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ρ,total</t>
+        </is>
+      </c>
+      <c r="L103" s="227">
+        <f>$L$102/($L$39*$L$38)*100</f>
+      </c>
+      <c r="M103" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="N103" s="232">
+        <f>IF($L$103&gt;4,"Rever: taxa &gt; 4% – aumentar seção",IF($L$103&lt;0.4,"Rever: taxa &lt; 0,4%","Ok"))</f>
+      </c>
+      <c r="O103" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Taxa total (pilar: 0,4% a 4%; 8% na emenda).</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="K104" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a,h,mín</t>
+        </is>
+      </c>
+      <c r="L104" s="227">
+        <f>MAX(2,$L$42/10,1.2*$L$36/10)</f>
+      </c>
+      <c r="M104" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O104" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mínimo: 2 cm, Ø,l e 1,2·d,máx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="K105" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a,h</t>
+        </is>
+      </c>
+      <c r="L105" s="227">
+        <f>IF($L$100&lt;=1,0,($L$39-2*$L$40-2*$L$41/10-$L$100*$L$42/10)/($L$100-1))</f>
+      </c>
+      <c r="M105" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="N105" s="232">
+        <f>IF($L$105&lt;$L$104,"Não cabe: aumentar b ou Ø,l",IF($L$105&gt;40,"Rever: espaço &gt; 40 cm","Ok"))</f>
+      </c>
+      <c r="O105" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espaço livre entre barras da mesma face.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="K107" s="221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 . ESTRIBOS – FORÇA CORTANTE (Modelo I, NBR 6118)</t>
+        </is>
+      </c>
+      <c r="L107" s="221"/>
+      <c r="M107" s="221"/>
+      <c r="N107" s="221"/>
+      <c r="O107" s="221"/>
+      <c r="P107" s="221"/>
+      <c r="Q107" s="221"/>
+      <c r="R107" s="221"/>
+      <c r="S107" s="221"/>
+      <c r="T107" s="221"/>
+    </row>
+    <row r="109" ht="32" customHeight="1">
+      <c r="K109" s="220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vsd ≤ VRd2 (biela) e Vsd ≤ Vc0 + Vsw. O espaçamento adotado é o menor entre o calculado, o máximo de viga (0,6·d ≤ 30 cm ou 0,3·d ≤ 20 cm) e o máximo de pilar (20 cm, b, 12·Ø,l).</t>
+        </is>
+      </c>
+      <c r="L109" s="220"/>
+      <c r="M109" s="220"/>
+      <c r="N109" s="220"/>
+      <c r="O109" s="220"/>
+      <c r="P109" s="220"/>
+      <c r="Q109" s="220"/>
+      <c r="R109" s="220"/>
+      <c r="S109" s="220"/>
+      <c r="T109" s="220"/>
+    </row>
+    <row r="110">
+      <c r="K110" s="222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.1 Biela e parcela do concreto</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="K111" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vsd</t>
+        </is>
+      </c>
+      <c r="L111" s="227">
+        <f>$L$48*$L$29</f>
+      </c>
+      <c r="M111" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kN</t>
+        </is>
+      </c>
+      <c r="O111" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cortante de cálculo (γf·Vk).</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="K112" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VRd2</t>
+        </is>
+      </c>
+      <c r="L112" s="227">
+        <f>0.27*(1-$L$33/250)*$L$62/10*$L$39*$L$65</f>
+      </c>
+      <c r="M112" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kN</t>
+        </is>
+      </c>
+      <c r="N112" s="232">
+        <f>IF($L$111&lt;=$L$112,"Ok","Aumentar seção ou fck")</f>
+      </c>
+      <c r="O112" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistência da biela comprimida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="K113" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fctm</t>
+        </is>
+      </c>
+      <c r="L113" s="227">
+        <f>0.3*$L$33^(2/3)</f>
+      </c>
+      <c r="M113" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPa</t>
+        </is>
+      </c>
+      <c r="O113" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistência média à tração.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="K114" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fctd</t>
+        </is>
+      </c>
+      <c r="L114" s="227">
+        <f>0.7*$L$113/$L$30</f>
+      </c>
+      <c r="M114" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPa</t>
+        </is>
+      </c>
+      <c r="O114" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistência de cálculo à tração (fctk,inf/γc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="K115" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vc0</t>
+        </is>
+      </c>
+      <c r="L115" s="227">
+        <f>0.6*$L$114/10*$L$39*$L$65</f>
+      </c>
+      <c r="M115" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kN</t>
+        </is>
+      </c>
+      <c r="O115" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parcela resistida pelo concreto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="K116" s="222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.2 Armadura transversal</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="K117" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fywd</t>
+        </is>
+      </c>
+      <c r="L117" s="227">
+        <f>MIN($L$35/$L$31,435)</f>
+      </c>
+      <c r="M117" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPa</t>
+        </is>
+      </c>
+      <c r="O117" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistência de cálculo do estribo (≤ 435 MPa).</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="K118" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vsw</t>
+        </is>
+      </c>
+      <c r="L118" s="227">
+        <f>MAX(0,$L$111-$L$115)</f>
+      </c>
+      <c r="M118" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kN</t>
+        </is>
+      </c>
+      <c r="O118" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parcela a ser resistida pelos estribos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="K119" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asw,calc</t>
+        </is>
+      </c>
+      <c r="L119" s="227">
+        <f>$L$118/(0.9*$L$65*$L$117/10)*100</f>
+      </c>
+      <c r="M119" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²/m</t>
+        </is>
+      </c>
+      <c r="O119" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asw/s = Vsw/(0,9·d·fywd).</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="K120" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asw,mín</t>
+        </is>
+      </c>
+      <c r="L120" s="227">
+        <f>0.2*$L$113/$L$35*$L$39*100</f>
+      </c>
+      <c r="M120" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²/m</t>
+        </is>
+      </c>
+      <c r="O120" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mínima: ρsw = 0,2·fctm/fywk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="K121" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asw</t>
+        </is>
+      </c>
+      <c r="L121" s="227">
+        <f>MAX($L$119,$L$120)</f>
+      </c>
+      <c r="M121" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²/m</t>
+        </is>
+      </c>
+      <c r="O121" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura transversal adotada (todos os ramos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="K122" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s,calc</t>
+        </is>
+      </c>
+      <c r="L122" s="227">
+        <f>IF($L$121=0,999,$L$43*PI()*($L$41/10)^2/4/$L$121*100)</f>
+      </c>
+      <c r="M122" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O122" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espaçamento pela armadura calculada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="K123" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s,máx,v</t>
+        </is>
+      </c>
+      <c r="L123" s="227">
+        <f>IF($L$111&lt;=0.67*$L$112,MIN(0.6*$L$65,30),MIN(0.3*$L$65,20))</f>
+      </c>
+      <c r="M123" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O123" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Máximo de viga (NBR 6118, 18.3.3.2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="K124" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s,máx,p</t>
+        </is>
+      </c>
+      <c r="L124" s="227">
+        <f>MIN(20,$L$39,$L$38,IF($L$34&gt;=500,12,25)*$L$42/10)</f>
+      </c>
+      <c r="M124" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O124" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Máximo de pilar: 20 cm, menor dimensão, 12·Ø,l (CA-50).</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="K125" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="L125" s="229">
+        <f>ROUNDDOWN(MIN($L$122,$L$123,$L$124),0)</f>
+      </c>
+      <c r="M125" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="N125" s="232">
+        <f>IF($L$125&lt;5,"s &lt; 5 cm – aumentar Ø,t ou ramos","Ok")</f>
+      </c>
+      <c r="O125" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espaçamento adotado (arredondado para baixo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="K126" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asw,ef</t>
+        </is>
+      </c>
+      <c r="L126" s="227">
+        <f>$L$43*PI()*($L$41/10)^2/4*100/$L$125</f>
+      </c>
+      <c r="M126" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²/m</t>
+        </is>
+      </c>
+      <c r="N126" s="232">
+        <f>IF($L$126&gt;=$L$121,"Ok","Rever")</f>
+      </c>
+      <c r="O126" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura efetiva com o espaçamento adotado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="K127" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ø,t,mín</t>
+        </is>
+      </c>
+      <c r="L127" s="227">
+        <f>MAX(5,$L$42/4)</f>
+      </c>
+      <c r="M127" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="N127" s="232">
+        <f>IF($L$41&gt;=$L$127,"Ok","Aumentar Ø,t")</f>
+      </c>
+      <c r="O127" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pilar: Ø,t ≥ 5 mm e ≥ Ø,l/4.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="33">
+    <mergeCell ref="K1:T1"/>
+    <mergeCell ref="K6:T6"/>
+    <mergeCell ref="K8:T8"/>
+    <mergeCell ref="K26:T26"/>
+    <mergeCell ref="K60:T60"/>
+    <mergeCell ref="K70:T70"/>
+    <mergeCell ref="K81:T81"/>
+    <mergeCell ref="K92:T92"/>
+    <mergeCell ref="K94:T94"/>
+    <mergeCell ref="K107:T107"/>
+    <mergeCell ref="K109:T109"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="O10:T10"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="L12:T12"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="L15:M15"/>
+    <mergeCell ref="L16:M16"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="R2:T2"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="O3:Q3"/>
+    <mergeCell ref="R3:T3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="O4:Q4"/>
+    <mergeCell ref="R4:T4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="N33 N42 N45 N68 N73 N84 N103 N105 N112 N125 N126 N127 N11 N13 N14 N15 N16 N17 N18">
+    <cfRule type="beginsWith" dxfId="6" priority="1" operator="beginsWith" text="Ok">
+      <formula>LEFT(N33,2)="Ok"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N33 N42 N45 N68 N73 N84 N103 N105 N112 N125 N126 N127 N11 N13 N14 N15 N16 N17 N18">
+    <cfRule type="beginsWith" dxfId="5" priority="2" operator="beginsWith" text="Não se aplica">
+      <formula>LEFT(N33,13)="Não se aplica"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L45">
+      <formula1>'CONTENÇÃO RÁPIDA'!$K$74:$K$76</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Dimensionamento pilar: painel congelado com As necessária, escolha da bitola, barras por face / espaçamento e OK / NÃO OK
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01STLw65tKW2EfXfQSwTwwMc
</commit_message>
<xml_diff>
--- a/3 - EMPUXO DE MUROS DE ARRIMO.xlsx
+++ b/3 - EMPUXO DE MUROS DE ARRIMO.xlsx
@@ -25,7 +25,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'CONTENÇÃO RÁPIDA'!$K$1:$T$259</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'DIMENSIONAMENTO PILAR'!$K$1:$T$127</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'DIMENSIONAMENTO PILAR'!$K$1:$T$138</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1" iterateCount="1000"/>
   <extLst>
@@ -1095,12 +1095,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.00000"/>
     <numFmt numFmtId="167" formatCode="0.000%"/>
     <numFmt numFmtId="168" formatCode="0.00"/>
+    <numFmt numFmtId="169" formatCode="&quot;Ø &quot;0.0&quot; mm&quot;"/>
   </numFmts>
   <fonts count="39" x14ac:knownFonts="1">
     <font>
@@ -2003,7 +2004,7 @@
     <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="242">
+  <cellXfs count="244">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2519,6 +2520,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="35" fillId="13" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -16124,19 +16131,19 @@
           <t xml:space="preserve">M11:M12</t>
         </is>
       </c>
-      <c r="L243" s="241" t="inlineStr">
+      <c r="L243" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">#REF! – referência apagada. São cópias antigas de M22/M23 (corretas). Podem ser apagadas.</t>
         </is>
       </c>
-      <c r="M243" s="241"/>
-      <c r="N243" s="241"/>
-      <c r="O243" s="241"/>
-      <c r="P243" s="241"/>
-      <c r="Q243" s="241"/>
-      <c r="R243" s="241"/>
-      <c r="S243" s="241"/>
-      <c r="T243" s="241"/>
+      <c r="M243" s="243"/>
+      <c r="N243" s="243"/>
+      <c r="O243" s="243"/>
+      <c r="P243" s="243"/>
+      <c r="Q243" s="243"/>
+      <c r="R243" s="243"/>
+      <c r="S243" s="243"/>
+      <c r="T243" s="243"/>
     </row>
     <row r="244" ht="32" customHeight="1">
       <c r="K244" s="238" t="inlineStr">
@@ -16144,19 +16151,19 @@
           <t xml:space="preserve">M22:M26</t>
         </is>
       </c>
-      <c r="L244" s="241" t="inlineStr">
+      <c r="L244" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">Carga no pilar só com o solo, sem a sobrecarga Sc (M30/M31 já incluem). Aqui: E (com Sc) e E,solo (sem Sc) – item 3.2.</t>
         </is>
       </c>
-      <c r="M244" s="241"/>
-      <c r="N244" s="241"/>
-      <c r="O244" s="241"/>
-      <c r="P244" s="241"/>
-      <c r="Q244" s="241"/>
-      <c r="R244" s="241"/>
-      <c r="S244" s="241"/>
-      <c r="T244" s="241"/>
+      <c r="M244" s="243"/>
+      <c r="N244" s="243"/>
+      <c r="O244" s="243"/>
+      <c r="P244" s="243"/>
+      <c r="Q244" s="243"/>
+      <c r="R244" s="243"/>
+      <c r="S244" s="243"/>
+      <c r="T244" s="243"/>
     </row>
     <row r="245" ht="17" customHeight="1">
       <c r="K245" s="238" t="inlineStr">
@@ -16164,19 +16171,19 @@
           <t xml:space="preserve">M26</t>
         </is>
       </c>
-      <c r="L245" s="241" t="inlineStr">
+      <c r="L245" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">Momento sem unidade: o resultado é em tf·m (base do pilar em balanço, sem Sc).</t>
         </is>
       </c>
-      <c r="M245" s="241"/>
-      <c r="N245" s="241"/>
-      <c r="O245" s="241"/>
-      <c r="P245" s="241"/>
-      <c r="Q245" s="241"/>
-      <c r="R245" s="241"/>
-      <c r="S245" s="241"/>
-      <c r="T245" s="241"/>
+      <c r="M245" s="243"/>
+      <c r="N245" s="243"/>
+      <c r="O245" s="243"/>
+      <c r="P245" s="243"/>
+      <c r="Q245" s="243"/>
+      <c r="R245" s="243"/>
+      <c r="S245" s="243"/>
+      <c r="T245" s="243"/>
     </row>
     <row r="246" ht="17" customHeight="1">
       <c r="K246" s="238" t="inlineStr">
@@ -16184,19 +16191,19 @@
           <t xml:space="preserve">M28</t>
         </is>
       </c>
-      <c r="L246" s="241" t="inlineStr">
+      <c r="L246" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">M25·M24/M27 com M27 = M25 → sempre igual a M24 (redundante, não é erro).</t>
         </is>
       </c>
-      <c r="M246" s="241"/>
-      <c r="N246" s="241"/>
-      <c r="O246" s="241"/>
-      <c r="P246" s="241"/>
-      <c r="Q246" s="241"/>
-      <c r="R246" s="241"/>
-      <c r="S246" s="241"/>
-      <c r="T246" s="241"/>
+      <c r="M246" s="243"/>
+      <c r="N246" s="243"/>
+      <c r="O246" s="243"/>
+      <c r="P246" s="243"/>
+      <c r="Q246" s="243"/>
+      <c r="R246" s="243"/>
+      <c r="S246" s="243"/>
+      <c r="T246" s="243"/>
     </row>
     <row r="247" ht="17" customHeight="1">
       <c r="K247" s="238" t="inlineStr">
@@ -16204,19 +16211,19 @@
           <t xml:space="preserve">M34</t>
         </is>
       </c>
-      <c r="L247" s="241" t="inlineStr">
+      <c r="L247" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">Só vale na cota 0 (usa H² na parcela uniforme). M36 é a fórmula certa para qualquer cota.</t>
         </is>
       </c>
-      <c r="M247" s="241"/>
-      <c r="N247" s="241"/>
-      <c r="O247" s="241"/>
-      <c r="P247" s="241"/>
-      <c r="Q247" s="241"/>
-      <c r="R247" s="241"/>
-      <c r="S247" s="241"/>
-      <c r="T247" s="241"/>
+      <c r="M247" s="243"/>
+      <c r="N247" s="243"/>
+      <c r="O247" s="243"/>
+      <c r="P247" s="243"/>
+      <c r="Q247" s="243"/>
+      <c r="R247" s="243"/>
+      <c r="S247" s="243"/>
+      <c r="T247" s="243"/>
     </row>
     <row r="248" ht="32" customHeight="1">
       <c r="K248" s="238" t="inlineStr">
@@ -16224,19 +16231,19 @@
           <t xml:space="preserve">M40</t>
         </is>
       </c>
-      <c r="L248" s="241" t="inlineStr">
+      <c r="L248" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">'Biapoiado' é na verdade engastado na base e apoiado no topo. Certo na cota 0 (−78,15 kN·m); para cota ≠ 0 os termos em x estão com sinal trocado e x²·Δp/2 aparece duplicado. Corrigido no item 4.1.</t>
         </is>
       </c>
-      <c r="M248" s="241"/>
-      <c r="N248" s="241"/>
-      <c r="O248" s="241"/>
-      <c r="P248" s="241"/>
-      <c r="Q248" s="241"/>
-      <c r="R248" s="241"/>
-      <c r="S248" s="241"/>
-      <c r="T248" s="241"/>
+      <c r="M248" s="243"/>
+      <c r="N248" s="243"/>
+      <c r="O248" s="243"/>
+      <c r="P248" s="243"/>
+      <c r="Q248" s="243"/>
+      <c r="R248" s="243"/>
+      <c r="S248" s="243"/>
+      <c r="T248" s="243"/>
     </row>
     <row r="249" ht="17" customHeight="1">
       <c r="K249" s="238" t="inlineStr">
@@ -16244,19 +16251,19 @@
           <t xml:space="preserve">P22:R27</t>
         </is>
       </c>
-      <c r="L249" s="241" t="inlineStr">
+      <c r="L249" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">Laje alveolar correta para o painel inferior (pressão na base × bw). O item 5 detalha todos os painéis.</t>
         </is>
       </c>
-      <c r="M249" s="241"/>
-      <c r="N249" s="241"/>
-      <c r="O249" s="241"/>
-      <c r="P249" s="241"/>
-      <c r="Q249" s="241"/>
-      <c r="R249" s="241"/>
-      <c r="S249" s="241"/>
-      <c r="T249" s="241"/>
+      <c r="M249" s="243"/>
+      <c r="N249" s="243"/>
+      <c r="O249" s="243"/>
+      <c r="P249" s="243"/>
+      <c r="Q249" s="243"/>
+      <c r="R249" s="243"/>
+      <c r="S249" s="243"/>
+      <c r="T249" s="243"/>
     </row>
     <row r="250" ht="17" customHeight="1">
       <c r="K250" s="238" t="inlineStr">
@@ -16264,19 +16271,19 @@
           <t xml:space="preserve">M24</t>
         </is>
       </c>
-      <c r="L250" s="241" t="inlineStr">
+      <c r="L250" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">kN → tf por ×0,1 (1 tf = 9,81 kN) fica ~2% abaixo do exato; mantido por ser a convenção usual.</t>
         </is>
       </c>
-      <c r="M250" s="241"/>
-      <c r="N250" s="241"/>
-      <c r="O250" s="241"/>
-      <c r="P250" s="241"/>
-      <c r="Q250" s="241"/>
-      <c r="R250" s="241"/>
-      <c r="S250" s="241"/>
-      <c r="T250" s="241"/>
+      <c r="M250" s="243"/>
+      <c r="N250" s="243"/>
+      <c r="O250" s="243"/>
+      <c r="P250" s="243"/>
+      <c r="Q250" s="243"/>
+      <c r="R250" s="243"/>
+      <c r="S250" s="243"/>
+      <c r="T250" s="243"/>
     </row>
     <row r="251" ht="32" customHeight="1">
       <c r="K251" s="238" t="inlineStr">
@@ -16284,19 +16291,19 @@
           <t xml:space="preserve">M8</t>
         </is>
       </c>
-      <c r="L251" s="241" t="inlineStr">
+      <c r="L251" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">Pilar travado no topo quase não se desloca: empuxo em repouso (K0) é mais realista que o ativo. Para φ = 18°: Ka = 0,53 e K0 = 0,69 (+31%). Use a entrada Empuxo (item 1.3).</t>
         </is>
       </c>
-      <c r="M251" s="241"/>
-      <c r="N251" s="241"/>
-      <c r="O251" s="241"/>
-      <c r="P251" s="241"/>
-      <c r="Q251" s="241"/>
-      <c r="R251" s="241"/>
-      <c r="S251" s="241"/>
-      <c r="T251" s="241"/>
+      <c r="M251" s="243"/>
+      <c r="N251" s="243"/>
+      <c r="O251" s="243"/>
+      <c r="P251" s="243"/>
+      <c r="Q251" s="243"/>
+      <c r="R251" s="243"/>
+      <c r="S251" s="243"/>
+      <c r="T251" s="243"/>
     </row>
     <row r="252">
       <c r="K252" s="222" t="inlineStr">
@@ -16311,19 +16318,19 @@
           <t xml:space="preserve">B20 / B28</t>
         </is>
       </c>
-      <c r="L253" s="241" t="inlineStr">
+      <c r="L253" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">#NUM! e #DIV/0!: a alvenaria pede 3,43 cm²/m e Ø8 em todo furo dá só 2,51 cm²/m → espaçamento '0 furos' e divisão por zero. Na prática: Ø8 não basta, usar Ø10 em todo furo (3,93 cm²/m).</t>
         </is>
       </c>
-      <c r="M253" s="241"/>
-      <c r="N253" s="241"/>
-      <c r="O253" s="241"/>
-      <c r="P253" s="241"/>
-      <c r="Q253" s="241"/>
-      <c r="R253" s="241"/>
-      <c r="S253" s="241"/>
-      <c r="T253" s="241"/>
+      <c r="M253" s="243"/>
+      <c r="N253" s="243"/>
+      <c r="O253" s="243"/>
+      <c r="P253" s="243"/>
+      <c r="Q253" s="243"/>
+      <c r="R253" s="243"/>
+      <c r="S253" s="243"/>
+      <c r="T253" s="243"/>
     </row>
     <row r="254" ht="17" customHeight="1">
       <c r="K254" s="238" t="inlineStr">
@@ -16331,19 +16338,19 @@
           <t xml:space="preserve">B8 / B9</t>
         </is>
       </c>
-      <c r="L254" s="241" t="inlineStr">
+      <c r="L254" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">Coesão e φ dão 0: NSPT (B4) = 0 não existe na tabela DADOS DO SOLO. Sem efeito, pois o Ka de B33 é digitado.</t>
         </is>
       </c>
-      <c r="M254" s="241"/>
-      <c r="N254" s="241"/>
-      <c r="O254" s="241"/>
-      <c r="P254" s="241"/>
-      <c r="Q254" s="241"/>
-      <c r="R254" s="241"/>
-      <c r="S254" s="241"/>
-      <c r="T254" s="241"/>
+      <c r="M254" s="243"/>
+      <c r="N254" s="243"/>
+      <c r="O254" s="243"/>
+      <c r="P254" s="243"/>
+      <c r="Q254" s="243"/>
+      <c r="R254" s="243"/>
+      <c r="S254" s="243"/>
+      <c r="T254" s="243"/>
     </row>
     <row r="255" ht="32" customHeight="1">
       <c r="K255" s="238" t="inlineStr">
@@ -16351,19 +16358,19 @@
           <t xml:space="preserve">B33</t>
         </is>
       </c>
-      <c r="L255" s="241" t="inlineStr">
+      <c r="L255" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">Ka = 0,36 digitado, sem ligação com φ. A aba usa 3 valores diferentes: 0,36 (B33), 0,528 (M8) e 0,75 (CÁLCULO FECHAMENTO).</t>
         </is>
       </c>
-      <c r="M255" s="241"/>
-      <c r="N255" s="241"/>
-      <c r="O255" s="241"/>
-      <c r="P255" s="241"/>
-      <c r="Q255" s="241"/>
-      <c r="R255" s="241"/>
-      <c r="S255" s="241"/>
-      <c r="T255" s="241"/>
+      <c r="M255" s="243"/>
+      <c r="N255" s="243"/>
+      <c r="O255" s="243"/>
+      <c r="P255" s="243"/>
+      <c r="Q255" s="243"/>
+      <c r="R255" s="243"/>
+      <c r="S255" s="243"/>
+      <c r="T255" s="243"/>
     </row>
     <row r="256" ht="32" customHeight="1">
       <c r="K256" s="238" t="inlineStr">
@@ -16371,19 +16378,19 @@
           <t xml:space="preserve">B24</t>
         </is>
       </c>
-      <c r="L256" s="241" t="inlineStr">
+      <c r="L256" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">Esbeltez do pilar usa a altura da alvenaria (1,75 m) em vez da do pilar (3,85 m). Com 3,85 m dá ≈ 25,7 &lt; 30 → segue 'Sim', por acaso.</t>
         </is>
       </c>
-      <c r="M256" s="241"/>
-      <c r="N256" s="241"/>
-      <c r="O256" s="241"/>
-      <c r="P256" s="241"/>
-      <c r="Q256" s="241"/>
-      <c r="R256" s="241"/>
-      <c r="S256" s="241"/>
-      <c r="T256" s="241"/>
+      <c r="M256" s="243"/>
+      <c r="N256" s="243"/>
+      <c r="O256" s="243"/>
+      <c r="P256" s="243"/>
+      <c r="Q256" s="243"/>
+      <c r="R256" s="243"/>
+      <c r="S256" s="243"/>
+      <c r="T256" s="243"/>
     </row>
     <row r="257" ht="32" customHeight="1">
       <c r="K257" s="238" t="inlineStr">
@@ -16391,19 +16398,19 @@
           <t xml:space="preserve">B52:B66</t>
         </is>
       </c>
-      <c r="L257" s="241" t="inlineStr">
+      <c r="L257" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">Pilar 20×30 não passa: Kc = 0,25 fora de tabela, Ks = 0,028 digitado não corresponde, As = 58 cm² (48 barras). Momento com (H/3 + 0,6) sem origem clara e sem Sc.</t>
         </is>
       </c>
-      <c r="M257" s="241"/>
-      <c r="N257" s="241"/>
-      <c r="O257" s="241"/>
-      <c r="P257" s="241"/>
-      <c r="Q257" s="241"/>
-      <c r="R257" s="241"/>
-      <c r="S257" s="241"/>
-      <c r="T257" s="241"/>
+      <c r="M257" s="243"/>
+      <c r="N257" s="243"/>
+      <c r="O257" s="243"/>
+      <c r="P257" s="243"/>
+      <c r="Q257" s="243"/>
+      <c r="R257" s="243"/>
+      <c r="S257" s="243"/>
+      <c r="T257" s="243"/>
     </row>
     <row r="258" ht="17" customHeight="1">
       <c r="K258" s="238" t="inlineStr">
@@ -16411,19 +16418,19 @@
           <t xml:space="preserve">B15</t>
         </is>
       </c>
-      <c r="L258" s="241" t="inlineStr">
+      <c r="L258" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">TABELAS LÍBANO com μ digitados para La/Lb = 0,91: se mudar H ou D, os coeficientes não se atualizam.</t>
         </is>
       </c>
-      <c r="M258" s="241"/>
-      <c r="N258" s="241"/>
-      <c r="O258" s="241"/>
-      <c r="P258" s="241"/>
-      <c r="Q258" s="241"/>
-      <c r="R258" s="241"/>
-      <c r="S258" s="241"/>
-      <c r="T258" s="241"/>
+      <c r="M258" s="243"/>
+      <c r="N258" s="243"/>
+      <c r="O258" s="243"/>
+      <c r="P258" s="243"/>
+      <c r="Q258" s="243"/>
+      <c r="R258" s="243"/>
+      <c r="S258" s="243"/>
+      <c r="T258" s="243"/>
     </row>
     <row r="259" ht="17" customHeight="1">
       <c r="K259" s="238" t="inlineStr">
@@ -16431,19 +16438,19 @@
           <t xml:space="preserve">B90</t>
         </is>
       </c>
-      <c r="L259" s="241" t="inlineStr">
+      <c r="L259" s="243" t="inlineStr">
         <is>
           <t xml:space="preserve">Peso da sapata fixo (1,2 × 1,0 × 0,5 m).</t>
         </is>
       </c>
-      <c r="M259" s="241"/>
-      <c r="N259" s="241"/>
-      <c r="O259" s="241"/>
-      <c r="P259" s="241"/>
-      <c r="Q259" s="241"/>
-      <c r="R259" s="241"/>
-      <c r="S259" s="241"/>
-      <c r="T259" s="241"/>
+      <c r="M259" s="243"/>
+      <c r="N259" s="243"/>
+      <c r="O259" s="243"/>
+      <c r="P259" s="243"/>
+      <c r="Q259" s="243"/>
+      <c r="R259" s="243"/>
+      <c r="S259" s="243"/>
+      <c r="T259" s="243"/>
     </row>
   </sheetData>
   <mergeCells count="59">
@@ -16536,7 +16543,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="K1:T127"/>
+  <dimension ref="K1:T138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="10" max="10" width="2.7109375" customWidth="1"/>
@@ -16571,63 +16578,67 @@
       </c>
       <c r="L2" s="239"/>
       <c r="M2" s="240">
-        <f>$L$100&amp;" Ø"&amp;$L$42&amp;" em cada face (simétrica)"</f>
+        <f>"As,nec = "&amp;FIXED($L$109,2)&amp;" cm²/face"</f>
       </c>
       <c r="N2" s="240"/>
-      <c r="O2" s="240">
-        <f>"As,ef = "&amp;FIXED($L$101,2)&amp;" cm²/face | total "&amp;FIXED($L$102,2)&amp;" cm²"</f>
-      </c>
-      <c r="P2" s="240"/>
+      <c r="O2" s="241">
+        <v>12.5</v>
+      </c>
+      <c r="P2" s="240">
+        <f>$L$111&amp;" barras em cada face ("&amp;FIXED($L$112,2)&amp;" cm²)"</f>
+      </c>
       <c r="Q2" s="240"/>
-      <c r="R2" s="240">
-        <f>"ρ = "&amp;FIXED($L$103,2)&amp;" % | "&amp;IF($L$105&lt;$L$104,"NÃO CABE","cabe na face")</f>
-      </c>
-      <c r="S2" s="240"/>
-      <c r="T2" s="240"/>
+      <c r="R2" s="240"/>
+      <c r="S2" s="242">
+        <f>IF($L$116&lt;$L$115,"NÃO OK – não cabe na face",IF($L$114&gt;4,"NÃO OK – taxa &gt; 4%",IF($L$42&lt;10,"NÃO OK – Ø &lt; 10 mm",IF($L$42&gt;$L$39*10/8,"NÃO OK – Ø &gt; b/8","OK"))))</f>
+      </c>
+      <c r="T2" s="242"/>
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="K3" s="239" t="inlineStr">
         <is>
-          <t xml:space="preserve">ESTRIBOS</t>
+          <t xml:space="preserve">ARMADURA TRANSVERSAL</t>
         </is>
       </c>
       <c r="L3" s="239"/>
       <c r="M3" s="240">
-        <f>"Ø"&amp;$L$41&amp;" c/"&amp;$L$125&amp;" ("&amp;$L$43&amp;" ramos)"</f>
+        <f>"Asw,nec = "&amp;FIXED($L$132,2)&amp;" cm²/m"</f>
       </c>
       <c r="N3" s="240"/>
-      <c r="O3" s="240">
-        <f>"Asw = "&amp;FIXED($L$121,2)&amp;" cm²/m"</f>
-      </c>
-      <c r="P3" s="240"/>
+      <c r="O3" s="241">
+        <v>6.3</v>
+      </c>
+      <c r="P3" s="240">
+        <f>"c/ "&amp;$L$136&amp;" cm ("&amp;$L$43&amp;" ramos) = "&amp;FIXED($L$137,2)&amp;" cm²/m"</f>
+      </c>
       <c r="Q3" s="240"/>
-      <c r="R3" s="240">
-        <f>"Vsd = "&amp;FIXED($L$111,1)&amp;" kN | VRd2 = "&amp;FIXED($L$112,1)&amp;" kN"</f>
-      </c>
-      <c r="S3" s="240"/>
-      <c r="T3" s="240"/>
+      <c r="R3" s="240"/>
+      <c r="S3" s="242">
+        <f>IF($L$122&gt;$L$123,"NÃO OK – biela: aumentar seção",IF($L$136&lt;5,"NÃO OK – s &lt; 5 cm: aumentar Ø",IF($L$41&lt;$L$138,"NÃO OK – Ø,t &lt; Ø,l/4","OK")))</f>
+      </c>
+      <c r="T3" s="242"/>
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="K4" s="239" t="inlineStr">
         <is>
-          <t xml:space="preserve">ESFORÇOS DE CÁLCULO</t>
+          <t xml:space="preserve">FLEXÃO / ESFORÇOS</t>
         </is>
       </c>
       <c r="L4" s="239"/>
       <c r="M4" s="240">
-        <f>"Md+ = "&amp;FIXED($L$72,2)&amp;" | Md− = "&amp;FIXED($L$83,2)&amp;" kN·m"</f>
+        <f>"Md+ = "&amp;FIXED($L$83,1)&amp;" | Md− = "&amp;FIXED($L$94,1)&amp;" kN·m"</f>
       </c>
       <c r="N4" s="240"/>
       <c r="O4" s="240">
-        <f>"Md,lim = "&amp;FIXED($L$67,2)&amp;" kN·m"</f>
+        <f>"Md,lim = "&amp;FIXED($L$78,1)&amp;" kN·m | Vsd = "&amp;FIXED($L$122,1)&amp;" kN ("&amp;$L$45&amp;")"</f>
       </c>
       <c r="P4" s="240"/>
       <c r="Q4" s="240"/>
-      <c r="R4" s="240">
-        <f>"Modelo: "&amp;$L$45&amp;" | seção "&amp;$L$39&amp;"×"&amp;$L$38</f>
-      </c>
-      <c r="S4" s="240"/>
-      <c r="T4" s="240"/>
+      <c r="R4" s="240"/>
+      <c r="S4" s="242">
+        <f>IF(MAX($L$83,$L$94)&gt;$L$78,"NÃO OK – arm. dupla: h ≥ "&amp;ROUNDUP($L$79+$L$75,0)&amp;" cm","OK – arm. simples")</f>
+      </c>
+      <c r="T4" s="242"/>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="K6" s="220" t="inlineStr">
@@ -16696,7 +16707,7 @@
         </is>
       </c>
       <c r="L11" s="236">
-        <f>"Md+ = "&amp;FIXED($L$72,1)&amp;" | Md− = "&amp;FIXED($L$83,1)</f>
+        <f>"Md+ = "&amp;FIXED($L$83,1)&amp;" | Md− = "&amp;FIXED($L$94,1)</f>
       </c>
       <c r="M11" s="236"/>
       <c r="N11" s="232">
@@ -16715,7 +16726,7 @@
         </is>
       </c>
       <c r="L12" s="234">
-        <f>IF(MAX($L$72,$L$83)&gt;$L$67,"⚠ Armadura dupla: a seção "&amp;$L$39&amp;"×"&amp;$L$38&amp;" é pequena para Md = "&amp;FIXED(MAX($L$72,$L$83),1)&amp;" kN·m. Para armadura simples use h ≥ "&amp;ROUNDUP($L$68+$L$64,0)&amp;" cm.","Flexão simples (sem a força normal): se o pilar tiver compressão relevante, confira a flexo-compressão no programa.")</f>
+        <f>IF(MAX($L$83,$L$94)&gt;$L$78,"⚠ Armadura dupla: a seção "&amp;$L$39&amp;"×"&amp;$L$38&amp;" é pequena para Md = "&amp;FIXED(MAX($L$83,$L$94),1)&amp;" kN·m. Para armadura simples use h ≥ "&amp;ROUNDUP($L$79+$L$75,0)&amp;" cm.","Flexão simples (sem a força normal): se o pilar tiver compressão relevante, confira a flexo-compressão no programa.")</f>
       </c>
       <c r="M12" s="234"/>
       <c r="N12" s="234"/>
@@ -16733,11 +16744,11 @@
         </is>
       </c>
       <c r="L13" s="236">
-        <f>$L$73</f>
+        <f>$L$84</f>
       </c>
       <c r="M13" s="236"/>
       <c r="N13" s="232">
-        <f>IF($L$72=0,"Não se aplica (M = 0)",IF($L$72&lt;=$L$67,"Ok","Arm. dupla – ver d,mín"))</f>
+        <f>IF($L$83=0,"Não se aplica (M = 0)",IF($L$83&lt;=$L$78,"Ok","Arm. dupla – ver d,mín"))</f>
       </c>
       <c r="O13" s="233" t="inlineStr">
         <is>
@@ -16752,11 +16763,11 @@
         </is>
       </c>
       <c r="L14" s="236">
-        <f>$L$84</f>
+        <f>$L$95</f>
       </c>
       <c r="M14" s="236"/>
       <c r="N14" s="232">
-        <f>IF($L$83=0,"Não se aplica (M = 0)",IF($L$83&lt;=$L$67,"Ok","Arm. dupla – ver d,mín"))</f>
+        <f>IF($L$94=0,"Não se aplica (M = 0)",IF($L$94&lt;=$L$78,"Ok","Arm. dupla – ver d,mín"))</f>
       </c>
       <c r="O14" s="233" t="inlineStr">
         <is>
@@ -16771,11 +16782,11 @@
         </is>
       </c>
       <c r="L15" s="236">
-        <f>$L$100&amp;" Ø"&amp;$L$42&amp;" ("&amp;FIXED($L$101,2)&amp;" cm²)"</f>
+        <f>$L$111&amp;" Ø"&amp;$L$42&amp;" ("&amp;FIXED($L$112,2)&amp;" cm²)"</f>
       </c>
       <c r="M15" s="236"/>
       <c r="N15" s="232">
-        <f>IF($L$105&lt;$L$104,"Não cabe: aumentar b ou Ø,l","Ok")</f>
+        <f>IF($L$116&lt;$L$115,"Não cabe: aumentar b ou Ø,l","Ok")</f>
       </c>
       <c r="O15" s="233" t="inlineStr">
         <is>
@@ -16790,11 +16801,11 @@
         </is>
       </c>
       <c r="L16" s="236">
-        <f>FIXED($L$103,2)&amp;" %"</f>
+        <f>FIXED($L$114,2)&amp;" %"</f>
       </c>
       <c r="M16" s="236"/>
       <c r="N16" s="232">
-        <f>IF($L$103&gt;4,"Rever: taxa &gt; 4%",IF($L$103&lt;0.4,"Rever: taxa &lt; 0,4%","Ok"))</f>
+        <f>IF($L$114&gt;4,"Rever: taxa &gt; 4%",IF($L$114&lt;0.4,"Rever: taxa &lt; 0,4%","Ok"))</f>
       </c>
       <c r="O16" s="233" t="inlineStr">
         <is>
@@ -16809,11 +16820,11 @@
         </is>
       </c>
       <c r="L17" s="236">
-        <f>FIXED($L$111,1)&amp;" ≤ "&amp;FIXED($L$112,1)&amp;" kN"</f>
+        <f>FIXED($L$122,1)&amp;" ≤ "&amp;FIXED($L$123,1)&amp;" kN"</f>
       </c>
       <c r="M17" s="236"/>
       <c r="N17" s="232">
-        <f>IF($L$111&lt;=$L$112,"Ok","Aumentar seção ou fck")</f>
+        <f>IF($L$122&lt;=$L$123,"Ok","Aumentar seção ou fck")</f>
       </c>
       <c r="O17" s="233" t="inlineStr">
         <is>
@@ -16828,11 +16839,11 @@
         </is>
       </c>
       <c r="L18" s="236">
-        <f>"Ø"&amp;$L$41&amp;" c/"&amp;$L$125&amp;" ("&amp;$L$43&amp;" ramos)"</f>
+        <f>"Ø"&amp;$L$41&amp;" c/"&amp;$L$136&amp;" ("&amp;$L$43&amp;" ramos)"</f>
       </c>
       <c r="M18" s="236"/>
       <c r="N18" s="232">
-        <f>IF($L$125&lt;5,"s &lt; 5 cm – aumentar Ø,t",IF($L$126&gt;=$L$121,"Ok","Rever"))</f>
+        <f>IF($L$136&lt;5,"s &lt; 5 cm – aumentar Ø,t",IF($L$137&gt;=$L$132,"Ok","Rever"))</f>
       </c>
       <c r="O18" s="233" t="inlineStr">
         <is>
@@ -17086,8 +17097,8 @@
           <t xml:space="preserve">Ø,t</t>
         </is>
       </c>
-      <c r="L41" s="224">
-        <v>6.3</v>
+      <c r="L41" s="227">
+        <f>$O$3</f>
       </c>
       <c r="M41" s="231" t="inlineStr">
         <is>
@@ -17096,7 +17107,7 @@
       </c>
       <c r="O41" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bitola do estribo.</t>
+          <t xml:space="preserve">Bitola do estribo – escolha no painel do topo (linha 3).</t>
         </is>
       </c>
     </row>
@@ -17106,8 +17117,8 @@
           <t xml:space="preserve">Ø,l</t>
         </is>
       </c>
-      <c r="L42" s="224">
-        <v>12.5</v>
+      <c r="L42" s="227">
+        <f>$O$2</f>
       </c>
       <c r="M42" s="231" t="inlineStr">
         <is>
@@ -17119,7 +17130,7 @@
       </c>
       <c r="O42" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bitola da armadura longitudinal.</t>
+          <t xml:space="preserve">Bitola longitudinal – escolha no painel do topo (linha 2).</t>
         </is>
       </c>
     </row>
@@ -17258,420 +17269,332 @@
     <row r="50">
       <c r="K50" s="222" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.5 Tabela ρ,mín (NBR 6118, tab. 17.3)</t>
+          <t xml:space="preserve">1.6 Bitolas disponíveis (lista do painel do topo)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="K51" s="235" t="inlineStr">
         <is>
+          <t xml:space="preserve">Ø (mm)</t>
+        </is>
+      </c>
+      <c r="L51" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Área (cm²)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="K52" s="224">
+        <v>5</v>
+      </c>
+      <c r="L52" s="228">
+        <f>PI()*(K52/10)^2/4</f>
+      </c>
+    </row>
+    <row r="53">
+      <c r="K53" s="224">
+        <v>6.3</v>
+      </c>
+      <c r="L53" s="228">
+        <f>PI()*(K53/10)^2/4</f>
+      </c>
+    </row>
+    <row r="54">
+      <c r="K54" s="224">
+        <v>8</v>
+      </c>
+      <c r="L54" s="228">
+        <f>PI()*(K54/10)^2/4</f>
+      </c>
+    </row>
+    <row r="55">
+      <c r="K55" s="224">
+        <v>10</v>
+      </c>
+      <c r="L55" s="228">
+        <f>PI()*(K55/10)^2/4</f>
+      </c>
+    </row>
+    <row r="56">
+      <c r="K56" s="224">
+        <v>12.5</v>
+      </c>
+      <c r="L56" s="228">
+        <f>PI()*(K56/10)^2/4</f>
+      </c>
+    </row>
+    <row r="57">
+      <c r="K57" s="224">
+        <v>16</v>
+      </c>
+      <c r="L57" s="228">
+        <f>PI()*(K57/10)^2/4</f>
+      </c>
+    </row>
+    <row r="58">
+      <c r="K58" s="224">
+        <v>20</v>
+      </c>
+      <c r="L58" s="228">
+        <f>PI()*(K58/10)^2/4</f>
+      </c>
+    </row>
+    <row r="59">
+      <c r="K59" s="224">
+        <v>25</v>
+      </c>
+      <c r="L59" s="228">
+        <f>PI()*(K59/10)^2/4</f>
+      </c>
+    </row>
+    <row r="60">
+      <c r="K60" s="224">
+        <v>32</v>
+      </c>
+      <c r="L60" s="228">
+        <f>PI()*(K60/10)^2/4</f>
+      </c>
+    </row>
+    <row r="61">
+      <c r="K61" s="222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.5 Tabela ρ,mín (NBR 6118, tab. 17.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="K62" s="235" t="inlineStr">
+        <is>
           <t xml:space="preserve">fck (MPa)</t>
         </is>
       </c>
-      <c r="L51" s="235" t="inlineStr">
+      <c r="L62" s="235" t="inlineStr">
         <is>
           <t xml:space="preserve">ρ,mín (%)</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="K52" s="237">
+    <row r="63">
+      <c r="K63" s="237">
         <v>20</v>
       </c>
-      <c r="L52" s="226">
+      <c r="L63" s="226">
         <v>0.15</v>
       </c>
     </row>
-    <row r="53">
-      <c r="K53" s="237">
+    <row r="64">
+      <c r="K64" s="237">
         <v>25</v>
       </c>
-      <c r="L53" s="226">
+      <c r="L64" s="226">
         <v>0.15</v>
       </c>
     </row>
-    <row r="54">
-      <c r="K54" s="237">
+    <row r="65">
+      <c r="K65" s="237">
         <v>30</v>
       </c>
-      <c r="L54" s="226">
+      <c r="L65" s="226">
         <v>0.15</v>
       </c>
     </row>
-    <row r="55">
-      <c r="K55" s="237">
+    <row r="66">
+      <c r="K66" s="237">
         <v>35</v>
       </c>
-      <c r="L55" s="226">
+      <c r="L66" s="226">
         <v>0.164</v>
       </c>
     </row>
-    <row r="56">
-      <c r="K56" s="237">
+    <row r="67">
+      <c r="K67" s="237">
         <v>40</v>
       </c>
-      <c r="L56" s="226">
+      <c r="L67" s="226">
         <v>0.179</v>
       </c>
     </row>
-    <row r="57">
-      <c r="K57" s="237">
+    <row r="68">
+      <c r="K68" s="237">
         <v>45</v>
       </c>
-      <c r="L57" s="226">
+      <c r="L68" s="226">
         <v>0.194</v>
       </c>
     </row>
-    <row r="58">
-      <c r="K58" s="237">
+    <row r="69">
+      <c r="K69" s="237">
         <v>50</v>
       </c>
-      <c r="L58" s="226">
+      <c r="L69" s="226">
         <v>0.208</v>
       </c>
     </row>
-    <row r="60">
-      <c r="K60" s="221" t="inlineStr">
+    <row r="71">
+      <c r="K71" s="221" t="inlineStr">
         <is>
           <t xml:space="preserve">2 . PARÂMETROS DE CÁLCULO</t>
         </is>
       </c>
-      <c r="L60" s="221"/>
-      <c r="M60" s="221"/>
-      <c r="N60" s="221"/>
-      <c r="O60" s="221"/>
-      <c r="P60" s="221"/>
-      <c r="Q60" s="221"/>
-      <c r="R60" s="221"/>
-      <c r="S60" s="221"/>
-      <c r="T60" s="221"/>
-    </row>
-    <row r="62">
-      <c r="K62" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fcd</t>
-        </is>
-      </c>
-      <c r="L62" s="227">
-        <f>$L$33/$L$30</f>
-      </c>
-      <c r="M62" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MPa</t>
-        </is>
-      </c>
-      <c r="O62" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Resistência de cálculo do concreto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="K63" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fyd</t>
-        </is>
-      </c>
-      <c r="L63" s="227">
-        <f>$L$34/$L$31</f>
-      </c>
-      <c r="M63" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MPa</t>
-        </is>
-      </c>
-      <c r="O63" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Resistência de cálculo do aço.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="K64" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">d'</t>
-        </is>
-      </c>
-      <c r="L64" s="227">
-        <f>$L$40+$L$41/10+$L$42/20</f>
-      </c>
-      <c r="M64" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cm</t>
-        </is>
-      </c>
-      <c r="O64" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Distância da face ao eixo das barras (c + Ø,t + Ø,l/2).</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="K65" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">d</t>
-        </is>
-      </c>
-      <c r="L65" s="227">
-        <f>$L$38-$L$64</f>
-      </c>
-      <c r="M65" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cm</t>
-        </is>
-      </c>
-      <c r="O65" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Altura útil (h − d').</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="K66" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(x/d)lim</t>
-        </is>
-      </c>
-      <c r="L66" s="227">
-        <v>0.45</v>
-      </c>
-      <c r="M66" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="O66" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Limite da linha neutra para fck ≤ 50 MPa (ductilidade).</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="K67" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Md,lim</t>
-        </is>
-      </c>
-      <c r="L67" s="227">
-        <f>0.68*$L$39*$L$65^2*$L$62/10*$L$66*(1-0.4*$L$66)/100</f>
-      </c>
-      <c r="M67" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kN·m</t>
-        </is>
-      </c>
-      <c r="O67" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Maior momento de cálculo só com armadura simples.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="K68" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">d,mín</t>
-        </is>
-      </c>
-      <c r="L68" s="227">
-        <f>SQRT(MAX($L$46,$L$47)*$L$29*100/(0.68*$L$39*$L$62/10*$L$66*(1-0.4*$L$66)))</f>
-      </c>
-      <c r="M68" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cm</t>
-        </is>
-      </c>
-      <c r="N68" s="232">
-        <f>IF($L$65&gt;=$L$68,"Ok","Aumentar h para "&amp;ROUNDUP($L$68+$L$64,0)&amp;" cm (arm. simples)")</f>
-      </c>
-      <c r="O68" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Altura útil mínima para armadura simples com o maior momento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="K70" s="221" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 . FLEXÃO – SEÇÃO DO VÃO (M+)</t>
-        </is>
-      </c>
-      <c r="L70" s="221"/>
-      <c r="M70" s="221"/>
-      <c r="N70" s="221"/>
-      <c r="O70" s="221"/>
-      <c r="P70" s="221"/>
-      <c r="Q70" s="221"/>
-      <c r="R70" s="221"/>
-      <c r="S70" s="221"/>
-      <c r="T70" s="221"/>
-    </row>
-    <row r="72">
-      <c r="K72" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Md</t>
-        </is>
-      </c>
-      <c r="L72" s="227">
-        <f>$L$46*$L$29</f>
-      </c>
-      <c r="M72" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kN·m</t>
-        </is>
-      </c>
-      <c r="O72" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Momento de cálculo (γf·Mk).</t>
-        </is>
-      </c>
+      <c r="L71" s="221"/>
+      <c r="M71" s="221"/>
+      <c r="N71" s="221"/>
+      <c r="O71" s="221"/>
+      <c r="P71" s="221"/>
+      <c r="Q71" s="221"/>
+      <c r="R71" s="221"/>
+      <c r="S71" s="221"/>
+      <c r="T71" s="221"/>
     </row>
     <row r="73">
       <c r="K73" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tipo</t>
-        </is>
-      </c>
-      <c r="L73" s="230">
-        <f>IF($L$72=0,"Não se aplica (M = 0)",IF($L$72&lt;=$L$67,"Armadura simples","Armadura dupla"))</f>
+          <t xml:space="preserve">fcd</t>
+        </is>
+      </c>
+      <c r="L73" s="227">
+        <f>$L$33/$L$30</f>
       </c>
       <c r="M73" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="N73" s="232">
-        <f>IF($L$72=0,"Não se aplica (M = 0)",IF($L$72&lt;=$L$67,"Ok","Arm. dupla – ver d,mín (item 2)"))</f>
+          <t xml:space="preserve">MPa</t>
+        </is>
       </c>
       <c r="O73" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Simples se Md ≤ Md,lim; dupla se maior.</t>
+          <t xml:space="preserve">Resistência de cálculo do concreto.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="K74" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">x</t>
+          <t xml:space="preserve">fyd</t>
         </is>
       </c>
       <c r="L74" s="227">
-        <f>IF($L$72&lt;=$L$67,1.25*$L$65*(1-SQRT(MAX(0,1-$L$72*100/(0.425*$L$39*$L$65^2*$L$62/10)))),$L$66*$L$65)</f>
+        <f>$L$34/$L$31</f>
       </c>
       <c r="M74" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm</t>
+          <t xml:space="preserve">MPa</t>
         </is>
       </c>
       <c r="O74" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Profundidade da linha neutra.</t>
+          <t xml:space="preserve">Resistência de cálculo do aço.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="K75" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">x/d</t>
-        </is>
-      </c>
-      <c r="L75" s="228">
-        <f>IF($L$65=0,0,$L$74/$L$65)</f>
+          <t xml:space="preserve">d'</t>
+        </is>
+      </c>
+      <c r="L75" s="227">
+        <f>$L$40+$L$41/10+$L$42/20</f>
       </c>
       <c r="M75" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">cm</t>
         </is>
       </c>
       <c r="O75" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Posição relativa da linha neutra.</t>
+          <t xml:space="preserve">Distância da face ao eixo das barras (c + Ø,t + Ø,l/2).</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="K76" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Domínio</t>
-        </is>
-      </c>
-      <c r="L76" s="230">
-        <f>IF($L$72=0,"-",IF($L$75&lt;=0.259,"2","3"))</f>
+          <t xml:space="preserve">d</t>
+        </is>
+      </c>
+      <c r="L76" s="227">
+        <f>$L$38-$L$75</f>
       </c>
       <c r="M76" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">cm</t>
         </is>
       </c>
       <c r="O76" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Domínio de deformação.</t>
+          <t xml:space="preserve">Altura útil (h − d').</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="K77" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">σsc</t>
+          <t xml:space="preserve">(x/d)lim</t>
         </is>
       </c>
       <c r="L77" s="227">
-        <f>MIN($L$63,210000*0.0035*MAX(0,$L$74-$L$64)/MAX($L$74,0.001))</f>
+        <v>0.45</v>
       </c>
       <c r="M77" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">MPa</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O77" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tensão na armadura comprimida (Es = 210 GPa, εc = 3,5‰), só na armadura dupla.</t>
+          <t xml:space="preserve">Limite da linha neutra para fck ≤ 50 MPa (ductilidade).</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="K78" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">As,t</t>
+          <t xml:space="preserve">Md,lim</t>
         </is>
       </c>
       <c r="L78" s="227">
-        <f>IF($L$72&lt;=$L$67,$L$72*100/($L$63/10*($L$65-0.4*$L$74)),$L$67*100/($L$63/10*($L$65-0.4*$L$74))+($L$72-$L$67)*100/($L$63/10*($L$65-$L$64)))</f>
+        <f>0.68*$L$39*$L$76^2*$L$73/10*$L$77*(1-0.4*$L$77)/100</f>
       </c>
       <c r="M78" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm²</t>
+          <t xml:space="preserve">kN·m</t>
         </is>
       </c>
       <c r="O78" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Armadura tracionada – face externa.</t>
+          <t xml:space="preserve">Maior momento de cálculo só com armadura simples.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="K79" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">As,c</t>
+          <t xml:space="preserve">d,mín</t>
         </is>
       </c>
       <c r="L79" s="227">
-        <f>IF($L$72&lt;=$L$67,0,($L$72-$L$67)*100/($L$77/10*($L$65-$L$64)))</f>
+        <f>SQRT(MAX($L$46,$L$47)*$L$29*100/(0.68*$L$39*$L$73/10*$L$77*(1-0.4*$L$77)))</f>
       </c>
       <c r="M79" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm²</t>
-        </is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="N79" s="232">
+        <f>IF($L$76&gt;=$L$79,"Ok","Aumentar h para "&amp;ROUNDUP($L$79+$L$75,0)&amp;" cm (arm. simples)")</f>
       </c>
       <c r="O79" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Armadura comprimida – face do solo (0 na armadura simples).</t>
+          <t xml:space="preserve">Altura útil mínima para armadura simples com o maior momento.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="K81" s="221" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 . FLEXÃO – SEÇÃO DA BASE (M−)</t>
+          <t xml:space="preserve">3 . FLEXÃO – SEÇÃO DO VÃO (M+)</t>
         </is>
       </c>
       <c r="L81" s="221"/>
@@ -17691,7 +17614,7 @@
         </is>
       </c>
       <c r="L83" s="227">
-        <f>$L$47*$L$29</f>
+        <f>$L$46*$L$29</f>
       </c>
       <c r="M83" s="231" t="inlineStr">
         <is>
@@ -17711,7 +17634,7 @@
         </is>
       </c>
       <c r="L84" s="230">
-        <f>IF($L$83=0,"Não se aplica (M = 0)",IF($L$83&lt;=$L$67,"Armadura simples","Armadura dupla"))</f>
+        <f>IF($L$83=0,"Não se aplica (M = 0)",IF($L$83&lt;=$L$78,"Armadura simples","Armadura dupla"))</f>
       </c>
       <c r="M84" s="231" t="inlineStr">
         <is>
@@ -17719,7 +17642,7 @@
         </is>
       </c>
       <c r="N84" s="232">
-        <f>IF($L$83=0,"Não se aplica (M = 0)",IF($L$83&lt;=$L$67,"Ok","Arm. dupla – ver d,mín (item 2)"))</f>
+        <f>IF($L$83=0,"Não se aplica (M = 0)",IF($L$83&lt;=$L$78,"Ok","Arm. dupla – ver d,mín (item 2)"))</f>
       </c>
       <c r="O84" s="233" t="inlineStr">
         <is>
@@ -17734,7 +17657,7 @@
         </is>
       </c>
       <c r="L85" s="227">
-        <f>IF($L$83&lt;=$L$67,1.25*$L$65*(1-SQRT(MAX(0,1-$L$83*100/(0.425*$L$39*$L$65^2*$L$62/10)))),$L$66*$L$65)</f>
+        <f>IF($L$83&lt;=$L$78,1.25*$L$76*(1-SQRT(MAX(0,1-$L$83*100/(0.425*$L$39*$L$76^2*$L$73/10)))),$L$77*$L$76)</f>
       </c>
       <c r="M85" s="231" t="inlineStr">
         <is>
@@ -17754,7 +17677,7 @@
         </is>
       </c>
       <c r="L86" s="228">
-        <f>IF($L$65=0,0,$L$85/$L$65)</f>
+        <f>IF($L$76=0,0,$L$85/$L$76)</f>
       </c>
       <c r="M86" s="231" t="inlineStr">
         <is>
@@ -17794,7 +17717,7 @@
         </is>
       </c>
       <c r="L88" s="227">
-        <f>MIN($L$63,210000*0.0035*MAX(0,$L$85-$L$64)/MAX($L$85,0.001))</f>
+        <f>MIN($L$74,210000*0.0035*MAX(0,$L$85-$L$75)/MAX($L$85,0.001))</f>
       </c>
       <c r="M88" s="231" t="inlineStr">
         <is>
@@ -17814,7 +17737,7 @@
         </is>
       </c>
       <c r="L89" s="227">
-        <f>IF($L$83&lt;=$L$67,$L$83*100/($L$63/10*($L$65-0.4*$L$85)),$L$67*100/($L$63/10*($L$65-0.4*$L$85))+($L$83-$L$67)*100/($L$63/10*($L$65-$L$64)))</f>
+        <f>IF($L$83&lt;=$L$78,$L$83*100/($L$74/10*($L$76-0.4*$L$85)),$L$78*100/($L$74/10*($L$76-0.4*$L$85))+($L$83-$L$78)*100/($L$74/10*($L$76-$L$75)))</f>
       </c>
       <c r="M89" s="231" t="inlineStr">
         <is>
@@ -17823,7 +17746,7 @@
       </c>
       <c r="O89" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Armadura tracionada – face do solo.</t>
+          <t xml:space="preserve">Armadura tracionada – face externa.</t>
         </is>
       </c>
     </row>
@@ -17834,7 +17757,7 @@
         </is>
       </c>
       <c r="L90" s="227">
-        <f>IF($L$83&lt;=$L$67,0,($L$83-$L$67)*100/($L$88/10*($L$65-$L$64)))</f>
+        <f>IF($L$83&lt;=$L$78,0,($L$83-$L$78)*100/($L$88/10*($L$76-$L$75)))</f>
       </c>
       <c r="M90" s="231" t="inlineStr">
         <is>
@@ -17843,14 +17766,14 @@
       </c>
       <c r="O90" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Armadura comprimida – face externa (0 na armadura simples).</t>
+          <t xml:space="preserve">Armadura comprimida – face do solo (0 na armadura simples).</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="K92" s="221" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 . ARMADURA LONGITUDINAL SIMÉTRICA (mesma nas duas faces)</t>
+          <t xml:space="preserve">4 . FLEXÃO – SEÇÃO DA BASE (M−)</t>
         </is>
       </c>
       <c r="L92" s="221"/>
@@ -17863,150 +17786,157 @@
       <c r="S92" s="221"/>
       <c r="T92" s="221"/>
     </row>
-    <row r="94" ht="32" customHeight="1">
-      <c r="K94" s="220" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cada face recebe a maior entre: tração do vão, tração da base, compressão da armadura dupla, mínima de viga (por face) e metade da mínima de pilar (0,4% Ac no total). As mesmas barras seguem por toda a altura, cobrindo as duas seções.</t>
-        </is>
-      </c>
-      <c r="L94" s="220"/>
-      <c r="M94" s="220"/>
-      <c r="N94" s="220"/>
-      <c r="O94" s="220"/>
-      <c r="P94" s="220"/>
-      <c r="Q94" s="220"/>
-      <c r="R94" s="220"/>
-      <c r="S94" s="220"/>
-      <c r="T94" s="220"/>
+    <row r="94">
+      <c r="K94" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Md</t>
+        </is>
+      </c>
+      <c r="L94" s="227">
+        <f>$L$47*$L$29</f>
+      </c>
+      <c r="M94" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kN·m</t>
+        </is>
+      </c>
+      <c r="O94" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Momento de cálculo (γf·Mk).</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="K95" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">ρ,mín</t>
-        </is>
-      </c>
-      <c r="L95" s="228">
-        <f>VLOOKUP($L$33,$K$52:$L$58,2,TRUE)</f>
+          <t xml:space="preserve">Tipo</t>
+        </is>
+      </c>
+      <c r="L95" s="230">
+        <f>IF($L$94=0,"Não se aplica (M = 0)",IF($L$94&lt;=$L$78,"Armadura simples","Armadura dupla"))</f>
       </c>
       <c r="M95" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">%</t>
-        </is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N95" s="232">
+        <f>IF($L$94=0,"Não se aplica (M = 0)",IF($L$94&lt;=$L$78,"Ok","Arm. dupla – ver d,mín (item 2)"))</f>
       </c>
       <c r="O95" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Taxa mínima de flexão (tabela 1.5).</t>
+          <t xml:space="preserve">Simples se Md ≤ Md,lim; dupla se maior.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="K96" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">As,mín,v</t>
+          <t xml:space="preserve">x</t>
         </is>
       </c>
       <c r="L96" s="227">
-        <f>$L$95/100*$L$39*$L$38</f>
+        <f>IF($L$94&lt;=$L$78,1.25*$L$76*(1-SQRT(MAX(0,1-$L$94*100/(0.425*$L$39*$L$76^2*$L$73/10)))),$L$77*$L$76)</f>
       </c>
       <c r="M96" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm²</t>
+          <t xml:space="preserve">cm</t>
         </is>
       </c>
       <c r="O96" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mínima de viga, por face tracionada: ρ,mín·b·h.</t>
+          <t xml:space="preserve">Profundidade da linha neutra.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="K97" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">As,mín,p</t>
-        </is>
-      </c>
-      <c r="L97" s="227">
-        <f>MAX(0.15*$L$49*$L$29/($L$63/10),0.004*$L$39*$L$38)</f>
+          <t xml:space="preserve">x/d</t>
+        </is>
+      </c>
+      <c r="L97" s="228">
+        <f>IF($L$76=0,0,$L$96/$L$76)</f>
       </c>
       <c r="M97" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm²</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O97" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mínima de pilar, total: máx(0,15·Nd/fyd; 0,4%·Ac).</t>
+          <t xml:space="preserve">Posição relativa da linha neutra.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="K98" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">As,face</t>
-        </is>
-      </c>
-      <c r="L98" s="227">
-        <f>MAX($L$78,$L$79,$L$89,$L$90,$L$96,$L$97/2)</f>
+          <t xml:space="preserve">Domínio</t>
+        </is>
+      </c>
+      <c r="L98" s="230">
+        <f>IF($L$94=0,"-",IF($L$97&lt;=0.259,"2","3"))</f>
       </c>
       <c r="M98" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm²</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="O98" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Armadura necessária em cada face.</t>
+          <t xml:space="preserve">Domínio de deformação.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="K99" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">A,barra</t>
-        </is>
-      </c>
-      <c r="L99" s="228">
-        <f>PI()*($L$42/10)^2/4</f>
+          <t xml:space="preserve">σsc</t>
+        </is>
+      </c>
+      <c r="L99" s="227">
+        <f>MIN($L$74,210000*0.0035*MAX(0,$L$96-$L$75)/MAX($L$96,0.001))</f>
       </c>
       <c r="M99" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm²</t>
+          <t xml:space="preserve">MPa</t>
         </is>
       </c>
       <c r="O99" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Área de uma barra Ø,l.</t>
+          <t xml:space="preserve">Tensão na armadura comprimida (Es = 210 GPa, εc = 3,5‰), só na armadura dupla.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="K100" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">n</t>
-        </is>
-      </c>
-      <c r="L100" s="229">
-        <f>MAX(2,ROUNDUP($L$98/$L$99,0))</f>
+          <t xml:space="preserve">As,t</t>
+        </is>
+      </c>
+      <c r="L100" s="227">
+        <f>IF($L$94&lt;=$L$78,$L$94*100/($L$74/10*($L$76-0.4*$L$96)),$L$78*100/($L$74/10*($L$76-0.4*$L$96))+($L$94-$L$78)*100/($L$74/10*($L$76-$L$75)))</f>
       </c>
       <c r="M100" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">un</t>
+          <t xml:space="preserve">cm²</t>
         </is>
       </c>
       <c r="O100" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Barras em cada face (mínimo 2).</t>
+          <t xml:space="preserve">Armadura tracionada – face do solo.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="K101" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">As,ef</t>
+          <t xml:space="preserve">As,c</t>
         </is>
       </c>
       <c r="L101" s="227">
-        <f>$L$100*$L$99</f>
+        <f>IF($L$94&lt;=$L$78,0,($L$94-$L$78)*100/($L$99/10*($L$76-$L$75)))</f>
       </c>
       <c r="M101" s="231" t="inlineStr">
         <is>
@@ -18015,469 +17945,641 @@
       </c>
       <c r="O101" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Armadura efetiva em cada face.</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="K102" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">As,total</t>
-        </is>
-      </c>
-      <c r="L102" s="227">
-        <f>2*$L$101</f>
-      </c>
-      <c r="M102" s="231" t="inlineStr">
+          <t xml:space="preserve">Armadura comprimida – face externa (0 na armadura simples).</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="K103" s="221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 . ARMADURA LONGITUDINAL SIMÉTRICA (mesma nas duas faces)</t>
+        </is>
+      </c>
+      <c r="L103" s="221"/>
+      <c r="M103" s="221"/>
+      <c r="N103" s="221"/>
+      <c r="O103" s="221"/>
+      <c r="P103" s="221"/>
+      <c r="Q103" s="221"/>
+      <c r="R103" s="221"/>
+      <c r="S103" s="221"/>
+      <c r="T103" s="221"/>
+    </row>
+    <row r="105" ht="32" customHeight="1">
+      <c r="K105" s="220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cada face recebe a maior entre: tração do vão, tração da base, compressão da armadura dupla, mínima de viga (por face) e metade da mínima de pilar (0,4% Ac no total). As mesmas barras seguem por toda a altura, cobrindo as duas seções.</t>
+        </is>
+      </c>
+      <c r="L105" s="220"/>
+      <c r="M105" s="220"/>
+      <c r="N105" s="220"/>
+      <c r="O105" s="220"/>
+      <c r="P105" s="220"/>
+      <c r="Q105" s="220"/>
+      <c r="R105" s="220"/>
+      <c r="S105" s="220"/>
+      <c r="T105" s="220"/>
+    </row>
+    <row r="106">
+      <c r="K106" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ρ,mín</t>
+        </is>
+      </c>
+      <c r="L106" s="228">
+        <f>VLOOKUP($L$33,$K$63:$L$69,2,TRUE)</f>
+      </c>
+      <c r="M106" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="O106" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Taxa mínima de flexão (tabela 1.5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="K107" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As,mín,v</t>
+        </is>
+      </c>
+      <c r="L107" s="227">
+        <f>$L$106/100*$L$39*$L$38</f>
+      </c>
+      <c r="M107" s="231" t="inlineStr">
         <is>
           <t xml:space="preserve">cm²</t>
         </is>
       </c>
-      <c r="O102" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Armadura total na seção (duas faces).</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="K103" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ρ,total</t>
-        </is>
-      </c>
-      <c r="L103" s="227">
-        <f>$L$102/($L$39*$L$38)*100</f>
-      </c>
-      <c r="M103" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">%</t>
-        </is>
-      </c>
-      <c r="N103" s="232">
-        <f>IF($L$103&gt;4,"Rever: taxa &gt; 4% – aumentar seção",IF($L$103&lt;0.4,"Rever: taxa &lt; 0,4%","Ok"))</f>
-      </c>
-      <c r="O103" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Taxa total (pilar: 0,4% a 4%; 8% na emenda).</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="K104" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a,h,mín</t>
-        </is>
-      </c>
-      <c r="L104" s="227">
-        <f>MAX(2,$L$42/10,1.2*$L$36/10)</f>
-      </c>
-      <c r="M104" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cm</t>
-        </is>
-      </c>
-      <c r="O104" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mínimo: 2 cm, Ø,l e 1,2·d,máx.</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="K105" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a,h</t>
-        </is>
-      </c>
-      <c r="L105" s="227">
-        <f>IF($L$100&lt;=1,0,($L$39-2*$L$40-2*$L$41/10-$L$100*$L$42/10)/($L$100-1))</f>
-      </c>
-      <c r="M105" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cm</t>
-        </is>
-      </c>
-      <c r="N105" s="232">
-        <f>IF($L$105&lt;$L$104,"Não cabe: aumentar b ou Ø,l",IF($L$105&gt;40,"Rever: espaço &gt; 40 cm","Ok"))</f>
-      </c>
-      <c r="O105" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Espaço livre entre barras da mesma face.</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="K107" s="221" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 . ESTRIBOS – FORÇA CORTANTE (Modelo I, NBR 6118)</t>
-        </is>
-      </c>
-      <c r="L107" s="221"/>
-      <c r="M107" s="221"/>
-      <c r="N107" s="221"/>
-      <c r="O107" s="221"/>
-      <c r="P107" s="221"/>
-      <c r="Q107" s="221"/>
-      <c r="R107" s="221"/>
-      <c r="S107" s="221"/>
-      <c r="T107" s="221"/>
-    </row>
-    <row r="109" ht="32" customHeight="1">
-      <c r="K109" s="220" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vsd ≤ VRd2 (biela) e Vsd ≤ Vc0 + Vsw. O espaçamento adotado é o menor entre o calculado, o máximo de viga (0,6·d ≤ 30 cm ou 0,3·d ≤ 20 cm) e o máximo de pilar (20 cm, b, 12·Ø,l).</t>
-        </is>
-      </c>
-      <c r="L109" s="220"/>
-      <c r="M109" s="220"/>
-      <c r="N109" s="220"/>
-      <c r="O109" s="220"/>
-      <c r="P109" s="220"/>
-      <c r="Q109" s="220"/>
-      <c r="R109" s="220"/>
-      <c r="S109" s="220"/>
-      <c r="T109" s="220"/>
+      <c r="O107" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mínima de viga, por face tracionada: ρ,mín·b·h.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="K108" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As,mín,p</t>
+        </is>
+      </c>
+      <c r="L108" s="227">
+        <f>MAX(0.15*$L$49*$L$29/($L$74/10),0.004*$L$39*$L$38)</f>
+      </c>
+      <c r="M108" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²</t>
+        </is>
+      </c>
+      <c r="O108" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mínima de pilar, total: máx(0,15·Nd/fyd; 0,4%·Ac).</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="K109" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As,face</t>
+        </is>
+      </c>
+      <c r="L109" s="227">
+        <f>MAX($L$89,$L$90,$L$100,$L$101,$L$107,$L$108/2)</f>
+      </c>
+      <c r="M109" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²</t>
+        </is>
+      </c>
+      <c r="O109" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura necessária em cada face.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
-      <c r="K110" s="222" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6.1 Biela e parcela do concreto</t>
+      <c r="K110" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A,barra</t>
+        </is>
+      </c>
+      <c r="L110" s="228">
+        <f>PI()*($L$42/10)^2/4</f>
+      </c>
+      <c r="M110" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²</t>
+        </is>
+      </c>
+      <c r="O110" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Área de uma barra Ø,l.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="K111" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vsd</t>
-        </is>
-      </c>
-      <c r="L111" s="227">
-        <f>$L$48*$L$29</f>
+          <t xml:space="preserve">n</t>
+        </is>
+      </c>
+      <c r="L111" s="229">
+        <f>MAX(2,ROUNDUP($L$109/$L$110,0))</f>
       </c>
       <c r="M111" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">kN</t>
+          <t xml:space="preserve">un</t>
         </is>
       </c>
       <c r="O111" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cortante de cálculo (γf·Vk).</t>
+          <t xml:space="preserve">Barras em cada face (mínimo 2).</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="K112" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">VRd2</t>
+          <t xml:space="preserve">As,ef</t>
         </is>
       </c>
       <c r="L112" s="227">
-        <f>0.27*(1-$L$33/250)*$L$62/10*$L$39*$L$65</f>
+        <f>$L$111*$L$110</f>
       </c>
       <c r="M112" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">kN</t>
-        </is>
-      </c>
-      <c r="N112" s="232">
-        <f>IF($L$111&lt;=$L$112,"Ok","Aumentar seção ou fck")</f>
+          <t xml:space="preserve">cm²</t>
+        </is>
       </c>
       <c r="O112" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resistência da biela comprimida.</t>
+          <t xml:space="preserve">Armadura efetiva em cada face.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="K113" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">fctm</t>
+          <t xml:space="preserve">As,total</t>
         </is>
       </c>
       <c r="L113" s="227">
-        <f>0.3*$L$33^(2/3)</f>
+        <f>2*$L$112</f>
       </c>
       <c r="M113" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">MPa</t>
+          <t xml:space="preserve">cm²</t>
         </is>
       </c>
       <c r="O113" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resistência média à tração.</t>
+          <t xml:space="preserve">Armadura total na seção (duas faces).</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="K114" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">fctd</t>
+          <t xml:space="preserve">ρ,total</t>
         </is>
       </c>
       <c r="L114" s="227">
-        <f>0.7*$L$113/$L$30</f>
+        <f>$L$113/($L$39*$L$38)*100</f>
       </c>
       <c r="M114" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">MPa</t>
-        </is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="N114" s="232">
+        <f>IF($L$114&gt;4,"Rever: taxa &gt; 4% – aumentar seção",IF($L$114&lt;0.4,"Rever: taxa &lt; 0,4%","Ok"))</f>
       </c>
       <c r="O114" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resistência de cálculo à tração (fctk,inf/γc).</t>
+          <t xml:space="preserve">Taxa total (pilar: 0,4% a 4%; 8% na emenda).</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="K115" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vc0</t>
+          <t xml:space="preserve">a,h,mín</t>
         </is>
       </c>
       <c r="L115" s="227">
-        <f>0.6*$L$114/10*$L$39*$L$65</f>
+        <f>MAX(2,$L$42/10,1.2*$L$36/10)</f>
       </c>
       <c r="M115" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">kN</t>
+          <t xml:space="preserve">cm</t>
         </is>
       </c>
       <c r="O115" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parcela resistida pelo concreto.</t>
+          <t xml:space="preserve">Mínimo: 2 cm, Ø,l e 1,2·d,máx.</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="K116" s="222" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6.2 Armadura transversal</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="K117" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fywd</t>
-        </is>
-      </c>
-      <c r="L117" s="227">
-        <f>MIN($L$35/$L$31,435)</f>
-      </c>
-      <c r="M117" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MPa</t>
-        </is>
-      </c>
-      <c r="O117" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Resistência de cálculo do estribo (≤ 435 MPa).</t>
+      <c r="K116" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a,h</t>
+        </is>
+      </c>
+      <c r="L116" s="227">
+        <f>IF($L$111&lt;=1,0,($L$39-2*$L$40-2*$L$41/10-$L$111*$L$42/10)/($L$111-1))</f>
+      </c>
+      <c r="M116" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="N116" s="232">
+        <f>IF($L$116&lt;$L$115,"Não cabe: aumentar b ou Ø,l",IF($L$116&gt;40,"Rever: espaço &gt; 40 cm","Ok"))</f>
+      </c>
+      <c r="O116" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espaço livre entre barras da mesma face.</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="K118" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vsw</t>
-        </is>
-      </c>
-      <c r="L118" s="227">
-        <f>MAX(0,$L$111-$L$115)</f>
-      </c>
-      <c r="M118" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kN</t>
-        </is>
-      </c>
-      <c r="O118" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Parcela a ser resistida pelos estribos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="K119" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Asw,calc</t>
-        </is>
-      </c>
-      <c r="L119" s="227">
-        <f>$L$118/(0.9*$L$65*$L$117/10)*100</f>
-      </c>
-      <c r="M119" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cm²/m</t>
-        </is>
-      </c>
-      <c r="O119" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Asw/s = Vsw/(0,9·d·fywd).</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="K120" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Asw,mín</t>
-        </is>
-      </c>
-      <c r="L120" s="227">
-        <f>0.2*$L$113/$L$35*$L$39*100</f>
-      </c>
-      <c r="M120" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cm²/m</t>
-        </is>
-      </c>
-      <c r="O120" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mínima: ρsw = 0,2·fctm/fywk.</t>
-        </is>
-      </c>
+      <c r="K118" s="221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 . ESTRIBOS – FORÇA CORTANTE (Modelo I, NBR 6118)</t>
+        </is>
+      </c>
+      <c r="L118" s="221"/>
+      <c r="M118" s="221"/>
+      <c r="N118" s="221"/>
+      <c r="O118" s="221"/>
+      <c r="P118" s="221"/>
+      <c r="Q118" s="221"/>
+      <c r="R118" s="221"/>
+      <c r="S118" s="221"/>
+      <c r="T118" s="221"/>
+    </row>
+    <row r="120" ht="32" customHeight="1">
+      <c r="K120" s="220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vsd ≤ VRd2 (biela) e Vsd ≤ Vc0 + Vsw. O espaçamento adotado é o menor entre o calculado, o máximo de viga (0,6·d ≤ 30 cm ou 0,3·d ≤ 20 cm) e o máximo de pilar (20 cm, b, 12·Ø,l).</t>
+        </is>
+      </c>
+      <c r="L120" s="220"/>
+      <c r="M120" s="220"/>
+      <c r="N120" s="220"/>
+      <c r="O120" s="220"/>
+      <c r="P120" s="220"/>
+      <c r="Q120" s="220"/>
+      <c r="R120" s="220"/>
+      <c r="S120" s="220"/>
+      <c r="T120" s="220"/>
     </row>
     <row r="121">
-      <c r="K121" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Asw</t>
-        </is>
-      </c>
-      <c r="L121" s="227">
-        <f>MAX($L$119,$L$120)</f>
-      </c>
-      <c r="M121" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cm²/m</t>
-        </is>
-      </c>
-      <c r="O121" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Armadura transversal adotada (todos os ramos).</t>
+      <c r="K121" s="222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.1 Biela e parcela do concreto</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="K122" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">s,calc</t>
+          <t xml:space="preserve">Vsd</t>
         </is>
       </c>
       <c r="L122" s="227">
-        <f>IF($L$121=0,999,$L$43*PI()*($L$41/10)^2/4/$L$121*100)</f>
+        <f>$L$48*$L$29</f>
       </c>
       <c r="M122" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm</t>
+          <t xml:space="preserve">kN</t>
         </is>
       </c>
       <c r="O122" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Espaçamento pela armadura calculada.</t>
+          <t xml:space="preserve">Cortante de cálculo (γf·Vk).</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="K123" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">s,máx,v</t>
+          <t xml:space="preserve">VRd2</t>
         </is>
       </c>
       <c r="L123" s="227">
-        <f>IF($L$111&lt;=0.67*$L$112,MIN(0.6*$L$65,30),MIN(0.3*$L$65,20))</f>
+        <f>0.27*(1-$L$33/250)*$L$73/10*$L$39*$L$76</f>
       </c>
       <c r="M123" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm</t>
-        </is>
+          <t xml:space="preserve">kN</t>
+        </is>
+      </c>
+      <c r="N123" s="232">
+        <f>IF($L$122&lt;=$L$123,"Ok","Aumentar seção ou fck")</f>
       </c>
       <c r="O123" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Máximo de viga (NBR 6118, 18.3.3.2).</t>
+          <t xml:space="preserve">Resistência da biela comprimida.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="K124" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">s,máx,p</t>
+          <t xml:space="preserve">fctm</t>
         </is>
       </c>
       <c r="L124" s="227">
-        <f>MIN(20,$L$39,$L$38,IF($L$34&gt;=500,12,25)*$L$42/10)</f>
+        <f>0.3*$L$33^(2/3)</f>
       </c>
       <c r="M124" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm</t>
+          <t xml:space="preserve">MPa</t>
         </is>
       </c>
       <c r="O124" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Máximo de pilar: 20 cm, menor dimensão, 12·Ø,l (CA-50).</t>
+          <t xml:space="preserve">Resistência média à tração.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="K125" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">s</t>
-        </is>
-      </c>
-      <c r="L125" s="229">
-        <f>ROUNDDOWN(MIN($L$122,$L$123,$L$124),0)</f>
+          <t xml:space="preserve">fctd</t>
+        </is>
+      </c>
+      <c r="L125" s="227">
+        <f>0.7*$L$124/$L$30</f>
       </c>
       <c r="M125" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm</t>
-        </is>
-      </c>
-      <c r="N125" s="232">
-        <f>IF($L$125&lt;5,"s &lt; 5 cm – aumentar Ø,t ou ramos","Ok")</f>
+          <t xml:space="preserve">MPa</t>
+        </is>
       </c>
       <c r="O125" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Espaçamento adotado (arredondado para baixo).</t>
+          <t xml:space="preserve">Resistência de cálculo à tração (fctk,inf/γc).</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="K126" s="223" t="inlineStr">
         <is>
+          <t xml:space="preserve">Vc0</t>
+        </is>
+      </c>
+      <c r="L126" s="227">
+        <f>0.6*$L$125/10*$L$39*$L$76</f>
+      </c>
+      <c r="M126" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kN</t>
+        </is>
+      </c>
+      <c r="O126" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parcela resistida pelo concreto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="K127" s="222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.2 Armadura transversal</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="K128" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fywd</t>
+        </is>
+      </c>
+      <c r="L128" s="227">
+        <f>MIN($L$35/$L$31,435)</f>
+      </c>
+      <c r="M128" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPa</t>
+        </is>
+      </c>
+      <c r="O128" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistência de cálculo do estribo (≤ 435 MPa).</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="K129" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vsw</t>
+        </is>
+      </c>
+      <c r="L129" s="227">
+        <f>MAX(0,$L$122-$L$126)</f>
+      </c>
+      <c r="M129" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kN</t>
+        </is>
+      </c>
+      <c r="O129" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parcela a ser resistida pelos estribos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="K130" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asw,calc</t>
+        </is>
+      </c>
+      <c r="L130" s="227">
+        <f>$L$129/(0.9*$L$76*$L$128/10)*100</f>
+      </c>
+      <c r="M130" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²/m</t>
+        </is>
+      </c>
+      <c r="O130" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asw/s = Vsw/(0,9·d·fywd).</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="K131" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asw,mín</t>
+        </is>
+      </c>
+      <c r="L131" s="227">
+        <f>0.2*$L$124/$L$35*$L$39*100</f>
+      </c>
+      <c r="M131" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²/m</t>
+        </is>
+      </c>
+      <c r="O131" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mínima: ρsw = 0,2·fctm/fywk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="K132" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asw</t>
+        </is>
+      </c>
+      <c r="L132" s="227">
+        <f>MAX($L$130,$L$131)</f>
+      </c>
+      <c r="M132" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²/m</t>
+        </is>
+      </c>
+      <c r="O132" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura transversal adotada (todos os ramos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="K133" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s,calc</t>
+        </is>
+      </c>
+      <c r="L133" s="227">
+        <f>IF($L$132=0,999,$L$43*PI()*($L$41/10)^2/4/$L$132*100)</f>
+      </c>
+      <c r="M133" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O133" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espaçamento pela armadura calculada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="K134" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s,máx,v</t>
+        </is>
+      </c>
+      <c r="L134" s="227">
+        <f>IF($L$122&lt;=0.67*$L$123,MIN(0.6*$L$76,30),MIN(0.3*$L$76,20))</f>
+      </c>
+      <c r="M134" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O134" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Máximo de viga (NBR 6118, 18.3.3.2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="K135" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s,máx,p</t>
+        </is>
+      </c>
+      <c r="L135" s="227">
+        <f>MIN(20,$L$39,$L$38,IF($L$34&gt;=500,12,25)*$L$42/10)</f>
+      </c>
+      <c r="M135" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O135" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Máximo de pilar: 20 cm, menor dimensão, 12·Ø,l (CA-50).</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="K136" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="L136" s="229">
+        <f>ROUNDDOWN(MIN($L$133,$L$134,$L$135),0)</f>
+      </c>
+      <c r="M136" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="N136" s="232">
+        <f>IF($L$136&lt;5,"s &lt; 5 cm – aumentar Ø,t ou ramos","Ok")</f>
+      </c>
+      <c r="O136" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Espaçamento adotado (arredondado para baixo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="K137" s="223" t="inlineStr">
+        <is>
           <t xml:space="preserve">Asw,ef</t>
         </is>
       </c>
-      <c r="L126" s="227">
-        <f>$L$43*PI()*($L$41/10)^2/4*100/$L$125</f>
-      </c>
-      <c r="M126" s="231" t="inlineStr">
+      <c r="L137" s="227">
+        <f>$L$43*PI()*($L$41/10)^2/4*100/$L$136</f>
+      </c>
+      <c r="M137" s="231" t="inlineStr">
         <is>
           <t xml:space="preserve">cm²/m</t>
         </is>
       </c>
-      <c r="N126" s="232">
-        <f>IF($L$126&gt;=$L$121,"Ok","Rever")</f>
-      </c>
-      <c r="O126" s="233" t="inlineStr">
+      <c r="N137" s="232">
+        <f>IF($L$137&gt;=$L$132,"Ok","Rever")</f>
+      </c>
+      <c r="O137" s="233" t="inlineStr">
         <is>
           <t xml:space="preserve">Armadura efetiva com o espaçamento adotado.</t>
         </is>
       </c>
     </row>
-    <row r="127">
-      <c r="K127" s="223" t="inlineStr">
+    <row r="138">
+      <c r="K138" s="223" t="inlineStr">
         <is>
           <t xml:space="preserve">Ø,t,mín</t>
         </is>
       </c>
-      <c r="L127" s="227">
+      <c r="L138" s="227">
         <f>MAX(5,$L$42/4)</f>
       </c>
-      <c r="M127" s="231" t="inlineStr">
+      <c r="M138" s="231" t="inlineStr">
         <is>
           <t xml:space="preserve">mm</t>
         </is>
       </c>
-      <c r="N127" s="232">
-        <f>IF($L$41&gt;=$L$127,"Ok","Aumentar Ø,t")</f>
-      </c>
-      <c r="O127" s="233" t="inlineStr">
+      <c r="N138" s="232">
+        <f>IF($L$41&gt;=$L$138,"Ok","Aumentar Ø,t")</f>
+      </c>
+      <c r="O138" s="233" t="inlineStr">
         <is>
           <t xml:space="preserve">Pilar: Ø,t ≥ 5 mm e ≥ Ø,l/4.</t>
         </is>
@@ -18489,13 +18591,13 @@
     <mergeCell ref="K6:T6"/>
     <mergeCell ref="K8:T8"/>
     <mergeCell ref="K26:T26"/>
-    <mergeCell ref="K60:T60"/>
-    <mergeCell ref="K70:T70"/>
+    <mergeCell ref="K71:T71"/>
     <mergeCell ref="K81:T81"/>
     <mergeCell ref="K92:T92"/>
-    <mergeCell ref="K94:T94"/>
-    <mergeCell ref="K107:T107"/>
-    <mergeCell ref="K109:T109"/>
+    <mergeCell ref="K103:T103"/>
+    <mergeCell ref="K105:T105"/>
+    <mergeCell ref="K118:T118"/>
+    <mergeCell ref="K120:T120"/>
     <mergeCell ref="L10:M10"/>
     <mergeCell ref="O10:T10"/>
     <mergeCell ref="L11:M11"/>
@@ -18508,30 +18610,33 @@
     <mergeCell ref="L18:M18"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="M2:N2"/>
-    <mergeCell ref="O2:Q2"/>
-    <mergeCell ref="R2:T2"/>
+    <mergeCell ref="P2:R2"/>
+    <mergeCell ref="S2:T2"/>
     <mergeCell ref="K3:L3"/>
     <mergeCell ref="M3:N3"/>
-    <mergeCell ref="O3:Q3"/>
-    <mergeCell ref="R3:T3"/>
+    <mergeCell ref="P3:R3"/>
+    <mergeCell ref="S3:T3"/>
     <mergeCell ref="K4:L4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="O4:Q4"/>
-    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="O4:R4"/>
+    <mergeCell ref="S4:T4"/>
   </mergeCells>
-  <conditionalFormatting sqref="N33 N42 N45 N68 N73 N84 N103 N105 N112 N125 N126 N127 N11 N13 N14 N15 N16 N17 N18">
+  <conditionalFormatting sqref="N33 N42 N45 N79 N84 N95 N114 N116 N123 N136 N137 N138 N11 N13 N14 N15 N16 N17 N18 S2 S3 S4">
     <cfRule type="beginsWith" dxfId="6" priority="1" operator="beginsWith" text="Ok">
       <formula>LEFT(N33,2)="Ok"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N33 N42 N45 N68 N73 N84 N103 N105 N112 N125 N126 N127 N11 N13 N14 N15 N16 N17 N18">
+  <conditionalFormatting sqref="N33 N42 N45 N79 N84 N95 N114 N116 N123 N136 N137 N138 N11 N13 N14 N15 N16 N17 N18 S2 S3 S4">
     <cfRule type="beginsWith" dxfId="5" priority="2" operator="beginsWith" text="Não se aplica">
       <formula>LEFT(N33,13)="Não se aplica"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L45">
       <formula1>'CONTENÇÃO RÁPIDA'!$K$74:$K$76</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="O2:O3">
+      <formula1>$K$52:$K$60</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>

</xml_diff>

<commit_message>
Dimensionamento pilar: taxa de aço (ρ e kg/m³) no painel congelado e seção 7
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01STLw65tKW2EfXfQSwTwwMc
</commit_message>
<xml_diff>
--- a/3 - EMPUXO DE MUROS DE ARRIMO.xlsx
+++ b/3 - EMPUXO DE MUROS DE ARRIMO.xlsx
@@ -25,7 +25,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'CONTENÇÃO RÁPIDA'!$K$1:$T$259</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'DIMENSIONAMENTO PILAR'!$K$1:$T$138</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'DIMENSIONAMENTO PILAR'!$K$1:$T$146</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1" iterateCount="1000"/>
   <extLst>
@@ -16543,7 +16543,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="K1:T138"/>
+  <dimension ref="K1:T146"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="10" max="10" width="2.7109375" customWidth="1"/>
@@ -16640,6 +16640,28 @@
       </c>
       <c r="T4" s="242"/>
     </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="K5" s="239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAXA DE AÇO</t>
+        </is>
+      </c>
+      <c r="L5" s="239"/>
+      <c r="M5" s="240">
+        <f>"ρ,long = "&amp;FIXED($L$114,2)&amp;" % (0,4% a 4%)"</f>
+      </c>
+      <c r="N5" s="240"/>
+      <c r="O5" s="240">
+        <f>"Longit. "&amp;FIXED($L$143,1)&amp;" + estribos "&amp;FIXED($L$145,1)&amp;" = "&amp;FIXED($L$146,1)&amp;" kg/m³"</f>
+      </c>
+      <c r="P5" s="240"/>
+      <c r="Q5" s="240"/>
+      <c r="R5" s="240"/>
+      <c r="S5" s="242">
+        <f>IF($L$114&gt;4,"NÃO OK – ρ &gt; 4%",IF($L$114&lt;0.4,"NÃO OK – ρ &lt; 0,4%","OK"))</f>
+      </c>
+      <c r="T5" s="242"/>
+    </row>
     <row r="6" ht="60" customHeight="1">
       <c r="K6" s="220" t="inlineStr">
         <is>
@@ -18585,8 +18607,124 @@
         </is>
       </c>
     </row>
+    <row r="140">
+      <c r="K140" s="221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7 . TAXA DE AÇO</t>
+        </is>
+      </c>
+      <c r="L140" s="221"/>
+      <c r="M140" s="221"/>
+      <c r="N140" s="221"/>
+      <c r="O140" s="221"/>
+      <c r="P140" s="221"/>
+      <c r="Q140" s="221"/>
+      <c r="R140" s="221"/>
+      <c r="S140" s="221"/>
+      <c r="T140" s="221"/>
+    </row>
+    <row r="142">
+      <c r="K142" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ρ,aço</t>
+        </is>
+      </c>
+      <c r="L142" s="224">
+        <v>0.785</v>
+      </c>
+      <c r="M142" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kg/m/cm²</t>
+        </is>
+      </c>
+      <c r="O142" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peso por metro de 1 cm² de barra (7850 kg/m³).</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="K143" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Longit.</t>
+        </is>
+      </c>
+      <c r="L143" s="227">
+        <f>$L$113*$L$142/($L$39*$L$38/10000)</f>
+      </c>
+      <c r="M143" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kg/m³</t>
+        </is>
+      </c>
+      <c r="O143" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura longitudinal (duas faces) por m³ de concreto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="K144" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">l,est</t>
+        </is>
+      </c>
+      <c r="L144" s="227">
+        <f>2*($L$39+$L$38)-8*$L$40+12</f>
+      </c>
+      <c r="M144" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O144" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comprimento de cada estribo (perímetro − cobrimentos + ganchos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="K145" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estribos</t>
+        </is>
+      </c>
+      <c r="L145" s="227">
+        <f>100/$L$136*$L$144/100*PI()*($L$41/10)^2/4*$L$142*$L$43/2/($L$39*$L$38/10000)</f>
+      </c>
+      <c r="M145" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kg/m³</t>
+        </is>
+      </c>
+      <c r="O145" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estribos por m³ de concreto (100/s estribos por metro).</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="K146" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
+      </c>
+      <c r="L146" s="227">
+        <f>$L$143+$L$145</f>
+      </c>
+      <c r="M146" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kg/m³</t>
+        </is>
+      </c>
+      <c r="O146" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Taxa total de aço do pilar.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="38">
     <mergeCell ref="K1:T1"/>
     <mergeCell ref="K6:T6"/>
     <mergeCell ref="K8:T8"/>
@@ -18598,6 +18736,7 @@
     <mergeCell ref="K105:T105"/>
     <mergeCell ref="K118:T118"/>
     <mergeCell ref="K120:T120"/>
+    <mergeCell ref="K140:T140"/>
     <mergeCell ref="L10:M10"/>
     <mergeCell ref="O10:T10"/>
     <mergeCell ref="L11:M11"/>
@@ -18620,13 +18759,17 @@
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="O4:R4"/>
     <mergeCell ref="S4:T4"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="M5:N5"/>
+    <mergeCell ref="O5:R5"/>
+    <mergeCell ref="S5:T5"/>
   </mergeCells>
-  <conditionalFormatting sqref="N33 N42 N45 N79 N84 N95 N114 N116 N123 N136 N137 N138 N11 N13 N14 N15 N16 N17 N18 S2 S3 S4">
+  <conditionalFormatting sqref="N33 N42 N45 N79 N84 N95 N114 N116 N123 N136 N137 N138 N11 N13 N14 N15 N16 N17 N18 S2 S3 S4 S5">
     <cfRule type="beginsWith" dxfId="6" priority="1" operator="beginsWith" text="Ok">
       <formula>LEFT(N33,2)="Ok"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N33 N42 N45 N79 N84 N95 N114 N116 N123 N136 N137 N138 N11 N13 N14 N15 N16 N17 N18 S2 S3 S4">
+  <conditionalFormatting sqref="N33 N42 N45 N79 N84 N95 N114 N116 N123 N136 N137 N138 N11 N13 N14 N15 N16 N17 N18 S2 S3 S4 S5">
     <cfRule type="beginsWith" dxfId="5" priority="2" operator="beginsWith" text="Não se aplica">
       <formula>LEFT(N33,13)="Não se aplica"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Dimensionamento pilar: status do espaçamento mostra espaço livre, mínimo e critério da NBR 6118 (18.4.2.2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01STLw65tKW2EfXfQSwTwwMc
</commit_message>
<xml_diff>
--- a/3 - EMPUXO DE MUROS DE ARRIMO.xlsx
+++ b/3 - EMPUXO DE MUROS DE ARRIMO.xlsx
@@ -25,7 +25,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'CONTENÇÃO RÁPIDA'!$K$1:$T$259</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'DIMENSIONAMENTO PILAR'!$K$1:$T$146</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'DIMENSIONAMENTO PILAR'!$K$1:$T$147</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1" iterateCount="1000"/>
   <extLst>
@@ -16543,7 +16543,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="K1:T146"/>
+  <dimension ref="K1:T147"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="10" max="10" width="2.7109375" customWidth="1"/>
@@ -16585,12 +16585,12 @@
         <v>12.5</v>
       </c>
       <c r="P2" s="240">
-        <f>$L$111&amp;" barras em cada face ("&amp;FIXED($L$112,2)&amp;" cm²)"</f>
+        <f>$L$111&amp;" barras em cada face ("&amp;FIXED($L$112,2)&amp;" cm²) | espaço livre "&amp;FIXED($L$117,2)&amp;" cm"</f>
       </c>
       <c r="Q2" s="240"/>
       <c r="R2" s="240"/>
       <c r="S2" s="242">
-        <f>IF($L$116&lt;$L$115,"NÃO OK – não cabe na face",IF($L$114&gt;4,"NÃO OK – taxa &gt; 4%",IF($L$42&lt;10,"NÃO OK – Ø &lt; 10 mm",IF($L$42&gt;$L$39*10/8,"NÃO OK – Ø &gt; b/8","OK"))))</f>
+        <f>IF($L$117&lt;$L$115,"NÃO OK – "&amp;"Espaço livre "&amp;FIXED($L$117,2)&amp;" &lt; "&amp;FIXED($L$115,2)&amp;" cm ("&amp;$L$116&amp;")",IF($L$114&gt;4,"NÃO OK – taxa &gt; 4%",IF($L$42&lt;10,"NÃO OK – Ø &lt; 10 mm",IF($L$42&gt;$L$39*10/8,"NÃO OK – Ø &gt; b/8","OK"))))</f>
       </c>
       <c r="T2" s="242"/>
     </row>
@@ -16602,19 +16602,19 @@
       </c>
       <c r="L3" s="239"/>
       <c r="M3" s="240">
-        <f>"Asw,nec = "&amp;FIXED($L$132,2)&amp;" cm²/m"</f>
+        <f>"Asw,nec = "&amp;FIXED($L$133,2)&amp;" cm²/m"</f>
       </c>
       <c r="N3" s="240"/>
       <c r="O3" s="241">
         <v>6.3</v>
       </c>
       <c r="P3" s="240">
-        <f>"c/ "&amp;$L$136&amp;" cm ("&amp;$L$43&amp;" ramos) = "&amp;FIXED($L$137,2)&amp;" cm²/m"</f>
+        <f>"c/ "&amp;$L$137&amp;" cm ("&amp;$L$43&amp;" ramos) = "&amp;FIXED($L$138,2)&amp;" cm²/m"</f>
       </c>
       <c r="Q3" s="240"/>
       <c r="R3" s="240"/>
       <c r="S3" s="242">
-        <f>IF($L$122&gt;$L$123,"NÃO OK – biela: aumentar seção",IF($L$136&lt;5,"NÃO OK – s &lt; 5 cm: aumentar Ø",IF($L$41&lt;$L$138,"NÃO OK – Ø,t &lt; Ø,l/4","OK")))</f>
+        <f>IF($L$123&gt;$L$124,"NÃO OK – biela: aumentar seção",IF($L$137&lt;5,"NÃO OK – s &lt; 5 cm: aumentar Ø",IF($L$41&lt;$L$139,"NÃO OK – Ø,t &lt; Ø,l/4","OK")))</f>
       </c>
       <c r="T3" s="242"/>
     </row>
@@ -16630,7 +16630,7 @@
       </c>
       <c r="N4" s="240"/>
       <c r="O4" s="240">
-        <f>"Md,lim = "&amp;FIXED($L$78,1)&amp;" kN·m | Vsd = "&amp;FIXED($L$122,1)&amp;" kN ("&amp;$L$45&amp;")"</f>
+        <f>"Md,lim = "&amp;FIXED($L$78,1)&amp;" kN·m | Vsd = "&amp;FIXED($L$123,1)&amp;" kN ("&amp;$L$45&amp;")"</f>
       </c>
       <c r="P4" s="240"/>
       <c r="Q4" s="240"/>
@@ -16652,7 +16652,7 @@
       </c>
       <c r="N5" s="240"/>
       <c r="O5" s="240">
-        <f>"Longit. "&amp;FIXED($L$143,1)&amp;" + estribos "&amp;FIXED($L$145,1)&amp;" = "&amp;FIXED($L$146,1)&amp;" kg/m³"</f>
+        <f>"Longit. "&amp;FIXED($L$144,1)&amp;" + estribos "&amp;FIXED($L$146,1)&amp;" = "&amp;FIXED($L$147,1)&amp;" kg/m³"</f>
       </c>
       <c r="P5" s="240"/>
       <c r="Q5" s="240"/>
@@ -16808,7 +16808,7 @@
       </c>
       <c r="M15" s="236"/>
       <c r="N15" s="232">
-        <f>IF($L$116&lt;$L$115,"Não cabe: aumentar b ou Ø,l","Ok")</f>
+        <f>IF($L$117&lt;$L$115,"Espaço livre "&amp;FIXED($L$117,2)&amp;" &lt; "&amp;FIXED($L$115,2)&amp;" cm ("&amp;$L$116&amp;")","Ok")</f>
       </c>
       <c r="O15" s="233" t="inlineStr">
         <is>
@@ -16842,11 +16842,11 @@
         </is>
       </c>
       <c r="L17" s="236">
-        <f>FIXED($L$122,1)&amp;" ≤ "&amp;FIXED($L$123,1)&amp;" kN"</f>
+        <f>FIXED($L$123,1)&amp;" ≤ "&amp;FIXED($L$124,1)&amp;" kN"</f>
       </c>
       <c r="M17" s="236"/>
       <c r="N17" s="232">
-        <f>IF($L$122&lt;=$L$123,"Ok","Aumentar seção ou fck")</f>
+        <f>IF($L$123&lt;=$L$124,"Ok","Aumentar seção ou fck")</f>
       </c>
       <c r="O17" s="233" t="inlineStr">
         <is>
@@ -16861,11 +16861,11 @@
         </is>
       </c>
       <c r="L18" s="236">
-        <f>"Ø"&amp;$L$41&amp;" c/"&amp;$L$136&amp;" ("&amp;$L$43&amp;" ramos)"</f>
+        <f>"Ø"&amp;$L$41&amp;" c/"&amp;$L$137&amp;" ("&amp;$L$43&amp;" ramos)"</f>
       </c>
       <c r="M18" s="236"/>
       <c r="N18" s="232">
-        <f>IF($L$136&lt;5,"s &lt; 5 cm – aumentar Ø,t",IF($L$137&gt;=$L$132,"Ok","Rever"))</f>
+        <f>IF($L$137&lt;5,"s &lt; 5 cm – aumentar Ø,t",IF($L$138&gt;=$L$133,"Ok","Rever"))</f>
       </c>
       <c r="O18" s="233" t="inlineStr">
         <is>
@@ -18202,143 +18202,143 @@
       </c>
       <c r="O115" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mínimo: 2 cm, Ø,l e 1,2·d,máx.</t>
+          <t xml:space="preserve">NBR 6118, 18.4.2.2: maior entre 2 cm, Ø,l e 1,2·d,máx.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="K116" s="223" t="inlineStr">
         <is>
+          <t xml:space="preserve">governa</t>
+        </is>
+      </c>
+      <c r="L116" s="230">
+        <f>IF($L$115=$L$42/10,"≥ Ø da barra",IF($L$115=2,"≥ 2 cm","≥ 1,2·d,máx"))</f>
+      </c>
+      <c r="M116" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O116" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Critério que define o espaço mínimo (brita 0: d,máx = 9,5 mm; brita 1: 19 mm).</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="K117" s="223" t="inlineStr">
+        <is>
           <t xml:space="preserve">a,h</t>
         </is>
       </c>
-      <c r="L116" s="227">
+      <c r="L117" s="227">
         <f>IF($L$111&lt;=1,0,($L$39-2*$L$40-2*$L$41/10-$L$111*$L$42/10)/($L$111-1))</f>
       </c>
-      <c r="M116" s="231" t="inlineStr">
+      <c r="M117" s="231" t="inlineStr">
         <is>
           <t xml:space="preserve">cm</t>
         </is>
       </c>
-      <c r="N116" s="232">
-        <f>IF($L$116&lt;$L$115,"Não cabe: aumentar b ou Ø,l",IF($L$116&gt;40,"Rever: espaço &gt; 40 cm","Ok"))</f>
-      </c>
-      <c r="O116" s="233" t="inlineStr">
+      <c r="N117" s="232">
+        <f>IF($L$117&lt;$L$115,"Espaço livre "&amp;FIXED($L$117,2)&amp;" &lt; "&amp;FIXED($L$115,2)&amp;" cm ("&amp;$L$116&amp;")",IF($L$117&gt;40,"Rever: espaço &gt; 40 cm","Ok"))</f>
+      </c>
+      <c r="O117" s="233" t="inlineStr">
         <is>
           <t xml:space="preserve">Espaço livre entre barras da mesma face.</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="K118" s="221" t="inlineStr">
+    <row r="119">
+      <c r="K119" s="221" t="inlineStr">
         <is>
           <t xml:space="preserve">6 . ESTRIBOS – FORÇA CORTANTE (Modelo I, NBR 6118)</t>
         </is>
       </c>
-      <c r="L118" s="221"/>
-      <c r="M118" s="221"/>
-      <c r="N118" s="221"/>
-      <c r="O118" s="221"/>
-      <c r="P118" s="221"/>
-      <c r="Q118" s="221"/>
-      <c r="R118" s="221"/>
-      <c r="S118" s="221"/>
-      <c r="T118" s="221"/>
-    </row>
-    <row r="120" ht="32" customHeight="1">
-      <c r="K120" s="220" t="inlineStr">
+      <c r="L119" s="221"/>
+      <c r="M119" s="221"/>
+      <c r="N119" s="221"/>
+      <c r="O119" s="221"/>
+      <c r="P119" s="221"/>
+      <c r="Q119" s="221"/>
+      <c r="R119" s="221"/>
+      <c r="S119" s="221"/>
+      <c r="T119" s="221"/>
+    </row>
+    <row r="121" ht="32" customHeight="1">
+      <c r="K121" s="220" t="inlineStr">
         <is>
           <t xml:space="preserve">Vsd ≤ VRd2 (biela) e Vsd ≤ Vc0 + Vsw. O espaçamento adotado é o menor entre o calculado, o máximo de viga (0,6·d ≤ 30 cm ou 0,3·d ≤ 20 cm) e o máximo de pilar (20 cm, b, 12·Ø,l).</t>
         </is>
       </c>
-      <c r="L120" s="220"/>
-      <c r="M120" s="220"/>
-      <c r="N120" s="220"/>
-      <c r="O120" s="220"/>
-      <c r="P120" s="220"/>
-      <c r="Q120" s="220"/>
-      <c r="R120" s="220"/>
-      <c r="S120" s="220"/>
-      <c r="T120" s="220"/>
-    </row>
-    <row r="121">
-      <c r="K121" s="222" t="inlineStr">
+      <c r="L121" s="220"/>
+      <c r="M121" s="220"/>
+      <c r="N121" s="220"/>
+      <c r="O121" s="220"/>
+      <c r="P121" s="220"/>
+      <c r="Q121" s="220"/>
+      <c r="R121" s="220"/>
+      <c r="S121" s="220"/>
+      <c r="T121" s="220"/>
+    </row>
+    <row r="122">
+      <c r="K122" s="222" t="inlineStr">
         <is>
           <t xml:space="preserve">6.1 Biela e parcela do concreto</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="K122" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vsd</t>
-        </is>
-      </c>
-      <c r="L122" s="227">
-        <f>$L$48*$L$29</f>
-      </c>
-      <c r="M122" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kN</t>
-        </is>
-      </c>
-      <c r="O122" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cortante de cálculo (γf·Vk).</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="K123" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">VRd2</t>
+          <t xml:space="preserve">Vsd</t>
         </is>
       </c>
       <c r="L123" s="227">
-        <f>0.27*(1-$L$33/250)*$L$73/10*$L$39*$L$76</f>
+        <f>$L$48*$L$29</f>
       </c>
       <c r="M123" s="231" t="inlineStr">
         <is>
           <t xml:space="preserve">kN</t>
         </is>
       </c>
-      <c r="N123" s="232">
-        <f>IF($L$122&lt;=$L$123,"Ok","Aumentar seção ou fck")</f>
-      </c>
       <c r="O123" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resistência da biela comprimida.</t>
+          <t xml:space="preserve">Cortante de cálculo (γf·Vk).</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="K124" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">fctm</t>
+          <t xml:space="preserve">VRd2</t>
         </is>
       </c>
       <c r="L124" s="227">
-        <f>0.3*$L$33^(2/3)</f>
+        <f>0.27*(1-$L$33/250)*$L$73/10*$L$39*$L$76</f>
       </c>
       <c r="M124" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">MPa</t>
-        </is>
+          <t xml:space="preserve">kN</t>
+        </is>
+      </c>
+      <c r="N124" s="232">
+        <f>IF($L$123&lt;=$L$124,"Ok","Aumentar seção ou fck")</f>
       </c>
       <c r="O124" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resistência média à tração.</t>
+          <t xml:space="preserve">Resistência da biela comprimida.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="K125" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">fctd</t>
+          <t xml:space="preserve">fctm</t>
         </is>
       </c>
       <c r="L125" s="227">
-        <f>0.7*$L$124/$L$30</f>
+        <f>0.3*$L$33^(2/3)</f>
       </c>
       <c r="M125" s="231" t="inlineStr">
         <is>
@@ -18347,105 +18347,105 @@
       </c>
       <c r="O125" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resistência de cálculo à tração (fctk,inf/γc).</t>
+          <t xml:space="preserve">Resistência média à tração.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="K126" s="223" t="inlineStr">
         <is>
+          <t xml:space="preserve">fctd</t>
+        </is>
+      </c>
+      <c r="L126" s="227">
+        <f>0.7*$L$125/$L$30</f>
+      </c>
+      <c r="M126" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPa</t>
+        </is>
+      </c>
+      <c r="O126" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistência de cálculo à tração (fctk,inf/γc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="K127" s="223" t="inlineStr">
+        <is>
           <t xml:space="preserve">Vc0</t>
         </is>
       </c>
-      <c r="L126" s="227">
-        <f>0.6*$L$125/10*$L$39*$L$76</f>
-      </c>
-      <c r="M126" s="231" t="inlineStr">
+      <c r="L127" s="227">
+        <f>0.6*$L$126/10*$L$39*$L$76</f>
+      </c>
+      <c r="M127" s="231" t="inlineStr">
         <is>
           <t xml:space="preserve">kN</t>
         </is>
       </c>
-      <c r="O126" s="233" t="inlineStr">
+      <c r="O127" s="233" t="inlineStr">
         <is>
           <t xml:space="preserve">Parcela resistida pelo concreto.</t>
         </is>
       </c>
     </row>
-    <row r="127">
-      <c r="K127" s="222" t="inlineStr">
+    <row r="128">
+      <c r="K128" s="222" t="inlineStr">
         <is>
           <t xml:space="preserve">6.2 Armadura transversal</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="K128" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fywd</t>
-        </is>
-      </c>
-      <c r="L128" s="227">
-        <f>MIN($L$35/$L$31,435)</f>
-      </c>
-      <c r="M128" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MPa</t>
-        </is>
-      </c>
-      <c r="O128" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Resistência de cálculo do estribo (≤ 435 MPa).</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="K129" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vsw</t>
+          <t xml:space="preserve">fywd</t>
         </is>
       </c>
       <c r="L129" s="227">
-        <f>MAX(0,$L$122-$L$126)</f>
+        <f>MIN($L$35/$L$31,435)</f>
       </c>
       <c r="M129" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">kN</t>
+          <t xml:space="preserve">MPa</t>
         </is>
       </c>
       <c r="O129" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parcela a ser resistida pelos estribos.</t>
+          <t xml:space="preserve">Resistência de cálculo do estribo (≤ 435 MPa).</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="K130" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asw,calc</t>
+          <t xml:space="preserve">Vsw</t>
         </is>
       </c>
       <c r="L130" s="227">
-        <f>$L$129/(0.9*$L$76*$L$128/10)*100</f>
+        <f>MAX(0,$L$123-$L$127)</f>
       </c>
       <c r="M130" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm²/m</t>
+          <t xml:space="preserve">kN</t>
         </is>
       </c>
       <c r="O130" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asw/s = Vsw/(0,9·d·fywd).</t>
+          <t xml:space="preserve">Parcela a ser resistida pelos estribos.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="K131" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asw,mín</t>
+          <t xml:space="preserve">Asw,calc</t>
         </is>
       </c>
       <c r="L131" s="227">
-        <f>0.2*$L$124/$L$35*$L$39*100</f>
+        <f>$L$130/(0.9*$L$76*$L$129/10)*100</f>
       </c>
       <c r="M131" s="231" t="inlineStr">
         <is>
@@ -18454,18 +18454,18 @@
       </c>
       <c r="O131" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mínima: ρsw = 0,2·fctm/fywk.</t>
+          <t xml:space="preserve">Asw/s = Vsw/(0,9·d·fywd).</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="K132" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asw</t>
+          <t xml:space="preserve">Asw,mín</t>
         </is>
       </c>
       <c r="L132" s="227">
-        <f>MAX($L$130,$L$131)</f>
+        <f>0.2*$L$125/$L$35*$L$39*100</f>
       </c>
       <c r="M132" s="231" t="inlineStr">
         <is>
@@ -18474,38 +18474,38 @@
       </c>
       <c r="O132" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Armadura transversal adotada (todos os ramos).</t>
+          <t xml:space="preserve">Mínima: ρsw = 0,2·fctm/fywk.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="K133" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">s,calc</t>
+          <t xml:space="preserve">Asw</t>
         </is>
       </c>
       <c r="L133" s="227">
-        <f>IF($L$132=0,999,$L$43*PI()*($L$41/10)^2/4/$L$132*100)</f>
+        <f>MAX($L$131,$L$132)</f>
       </c>
       <c r="M133" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm</t>
+          <t xml:space="preserve">cm²/m</t>
         </is>
       </c>
       <c r="O133" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Espaçamento pela armadura calculada.</t>
+          <t xml:space="preserve">Armadura transversal adotada (todos os ramos).</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="K134" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">s,máx,v</t>
+          <t xml:space="preserve">s,calc</t>
         </is>
       </c>
       <c r="L134" s="227">
-        <f>IF($L$122&lt;=0.67*$L$123,MIN(0.6*$L$76,30),MIN(0.3*$L$76,20))</f>
+        <f>IF($L$133=0,999,$L$43*PI()*($L$41/10)^2/4/$L$133*100)</f>
       </c>
       <c r="M134" s="231" t="inlineStr">
         <is>
@@ -18514,18 +18514,18 @@
       </c>
       <c r="O134" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Máximo de viga (NBR 6118, 18.3.3.2).</t>
+          <t xml:space="preserve">Espaçamento pela armadura calculada.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="K135" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">s,máx,p</t>
+          <t xml:space="preserve">s,máx,v</t>
         </is>
       </c>
       <c r="L135" s="227">
-        <f>MIN(20,$L$39,$L$38,IF($L$34&gt;=500,12,25)*$L$42/10)</f>
+        <f>IF($L$123&lt;=0.67*$L$124,MIN(0.6*$L$76,30),MIN(0.3*$L$76,20))</f>
       </c>
       <c r="M135" s="231" t="inlineStr">
         <is>
@@ -18534,190 +18534,210 @@
       </c>
       <c r="O135" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Máximo de pilar: 20 cm, menor dimensão, 12·Ø,l (CA-50).</t>
+          <t xml:space="preserve">Máximo de viga (NBR 6118, 18.3.3.2).</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="K136" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">s</t>
-        </is>
-      </c>
-      <c r="L136" s="229">
-        <f>ROUNDDOWN(MIN($L$133,$L$134,$L$135),0)</f>
+          <t xml:space="preserve">s,máx,p</t>
+        </is>
+      </c>
+      <c r="L136" s="227">
+        <f>MIN(20,$L$39,$L$38,IF($L$34&gt;=500,12,25)*$L$42/10)</f>
       </c>
       <c r="M136" s="231" t="inlineStr">
         <is>
           <t xml:space="preserve">cm</t>
         </is>
       </c>
-      <c r="N136" s="232">
-        <f>IF($L$136&lt;5,"s &lt; 5 cm – aumentar Ø,t ou ramos","Ok")</f>
-      </c>
       <c r="O136" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Espaçamento adotado (arredondado para baixo).</t>
+          <t xml:space="preserve">Máximo de pilar: 20 cm, menor dimensão, 12·Ø,l (CA-50).</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="K137" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asw,ef</t>
-        </is>
-      </c>
-      <c r="L137" s="227">
-        <f>$L$43*PI()*($L$41/10)^2/4*100/$L$136</f>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="L137" s="229">
+        <f>ROUNDDOWN(MIN($L$134,$L$135,$L$136),0)</f>
       </c>
       <c r="M137" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm²/m</t>
+          <t xml:space="preserve">cm</t>
         </is>
       </c>
       <c r="N137" s="232">
-        <f>IF($L$137&gt;=$L$132,"Ok","Rever")</f>
+        <f>IF($L$137&lt;5,"s &lt; 5 cm – aumentar Ø,t ou ramos","Ok")</f>
       </c>
       <c r="O137" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Armadura efetiva com o espaçamento adotado.</t>
+          <t xml:space="preserve">Espaçamento adotado (arredondado para baixo).</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="K138" s="223" t="inlineStr">
         <is>
+          <t xml:space="preserve">Asw,ef</t>
+        </is>
+      </c>
+      <c r="L138" s="227">
+        <f>$L$43*PI()*($L$41/10)^2/4*100/$L$137</f>
+      </c>
+      <c r="M138" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm²/m</t>
+        </is>
+      </c>
+      <c r="N138" s="232">
+        <f>IF($L$138&gt;=$L$133,"Ok","Rever")</f>
+      </c>
+      <c r="O138" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura efetiva com o espaçamento adotado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="K139" s="223" t="inlineStr">
+        <is>
           <t xml:space="preserve">Ø,t,mín</t>
         </is>
       </c>
-      <c r="L138" s="227">
+      <c r="L139" s="227">
         <f>MAX(5,$L$42/4)</f>
       </c>
-      <c r="M138" s="231" t="inlineStr">
+      <c r="M139" s="231" t="inlineStr">
         <is>
           <t xml:space="preserve">mm</t>
         </is>
       </c>
-      <c r="N138" s="232">
-        <f>IF($L$41&gt;=$L$138,"Ok","Aumentar Ø,t")</f>
-      </c>
-      <c r="O138" s="233" t="inlineStr">
+      <c r="N139" s="232">
+        <f>IF($L$41&gt;=$L$139,"Ok","Aumentar Ø,t")</f>
+      </c>
+      <c r="O139" s="233" t="inlineStr">
         <is>
           <t xml:space="preserve">Pilar: Ø,t ≥ 5 mm e ≥ Ø,l/4.</t>
         </is>
       </c>
     </row>
-    <row r="140">
-      <c r="K140" s="221" t="inlineStr">
+    <row r="141">
+      <c r="K141" s="221" t="inlineStr">
         <is>
           <t xml:space="preserve">7 . TAXA DE AÇO</t>
         </is>
       </c>
-      <c r="L140" s="221"/>
-      <c r="M140" s="221"/>
-      <c r="N140" s="221"/>
-      <c r="O140" s="221"/>
-      <c r="P140" s="221"/>
-      <c r="Q140" s="221"/>
-      <c r="R140" s="221"/>
-      <c r="S140" s="221"/>
-      <c r="T140" s="221"/>
-    </row>
-    <row r="142">
-      <c r="K142" s="223" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ρ,aço</t>
-        </is>
-      </c>
-      <c r="L142" s="224">
-        <v>0.785</v>
-      </c>
-      <c r="M142" s="231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kg/m/cm²</t>
-        </is>
-      </c>
-      <c r="O142" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Peso por metro de 1 cm² de barra (7850 kg/m³).</t>
-        </is>
-      </c>
+      <c r="L141" s="221"/>
+      <c r="M141" s="221"/>
+      <c r="N141" s="221"/>
+      <c r="O141" s="221"/>
+      <c r="P141" s="221"/>
+      <c r="Q141" s="221"/>
+      <c r="R141" s="221"/>
+      <c r="S141" s="221"/>
+      <c r="T141" s="221"/>
     </row>
     <row r="143">
       <c r="K143" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Longit.</t>
-        </is>
-      </c>
-      <c r="L143" s="227">
-        <f>$L$113*$L$142/($L$39*$L$38/10000)</f>
+          <t xml:space="preserve">ρ,aço</t>
+        </is>
+      </c>
+      <c r="L143" s="224">
+        <v>0.785</v>
       </c>
       <c r="M143" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">kg/m³</t>
+          <t xml:space="preserve">kg/m/cm²</t>
         </is>
       </c>
       <c r="O143" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Armadura longitudinal (duas faces) por m³ de concreto.</t>
+          <t xml:space="preserve">Peso por metro de 1 cm² de barra (7850 kg/m³).</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="K144" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">l,est</t>
+          <t xml:space="preserve">Longit.</t>
         </is>
       </c>
       <c r="L144" s="227">
-        <f>2*($L$39+$L$38)-8*$L$40+12</f>
+        <f>$L$113*$L$143/($L$39*$L$38/10000)</f>
       </c>
       <c r="M144" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm</t>
+          <t xml:space="preserve">kg/m³</t>
         </is>
       </c>
       <c r="O144" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comprimento de cada estribo (perímetro − cobrimentos + ganchos).</t>
+          <t xml:space="preserve">Armadura longitudinal (duas faces) por m³ de concreto.</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="K145" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Estribos</t>
+          <t xml:space="preserve">l,est</t>
         </is>
       </c>
       <c r="L145" s="227">
-        <f>100/$L$136*$L$144/100*PI()*($L$41/10)^2/4*$L$142*$L$43/2/($L$39*$L$38/10000)</f>
+        <f>2*($L$39+$L$38)-8*$L$40+12</f>
       </c>
       <c r="M145" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">kg/m³</t>
+          <t xml:space="preserve">cm</t>
         </is>
       </c>
       <c r="O145" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Estribos por m³ de concreto (100/s estribos por metro).</t>
+          <t xml:space="preserve">Comprimento de cada estribo (perímetro − cobrimentos + ganchos).</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="K146" s="223" t="inlineStr">
         <is>
+          <t xml:space="preserve">Estribos</t>
+        </is>
+      </c>
+      <c r="L146" s="227">
+        <f>100/$L$137*$L$145/100*PI()*($L$41/10)^2/4*$L$143*$L$43/2/($L$39*$L$38/10000)</f>
+      </c>
+      <c r="M146" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kg/m³</t>
+        </is>
+      </c>
+      <c r="O146" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estribos por m³ de concreto (100/s estribos por metro).</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="K147" s="223" t="inlineStr">
+        <is>
           <t xml:space="preserve">Total</t>
         </is>
       </c>
-      <c r="L146" s="227">
-        <f>$L$143+$L$145</f>
-      </c>
-      <c r="M146" s="231" t="inlineStr">
+      <c r="L147" s="227">
+        <f>$L$144+$L$146</f>
+      </c>
+      <c r="M147" s="231" t="inlineStr">
         <is>
           <t xml:space="preserve">kg/m³</t>
         </is>
       </c>
-      <c r="O146" s="233" t="inlineStr">
+      <c r="O147" s="233" t="inlineStr">
         <is>
           <t xml:space="preserve">Taxa total de aço do pilar.</t>
         </is>
@@ -18734,9 +18754,9 @@
     <mergeCell ref="K92:T92"/>
     <mergeCell ref="K103:T103"/>
     <mergeCell ref="K105:T105"/>
-    <mergeCell ref="K118:T118"/>
-    <mergeCell ref="K120:T120"/>
-    <mergeCell ref="K140:T140"/>
+    <mergeCell ref="K119:T119"/>
+    <mergeCell ref="K121:T121"/>
+    <mergeCell ref="K141:T141"/>
     <mergeCell ref="L10:M10"/>
     <mergeCell ref="O10:T10"/>
     <mergeCell ref="L11:M11"/>
@@ -18764,12 +18784,12 @@
     <mergeCell ref="O5:R5"/>
     <mergeCell ref="S5:T5"/>
   </mergeCells>
-  <conditionalFormatting sqref="N33 N42 N45 N79 N84 N95 N114 N116 N123 N136 N137 N138 N11 N13 N14 N15 N16 N17 N18 S2 S3 S4 S5">
+  <conditionalFormatting sqref="N33 N42 N45 N79 N84 N95 N114 N117 N124 N137 N138 N139 N11 N13 N14 N15 N16 N17 N18 S2 S3 S4 S5">
     <cfRule type="beginsWith" dxfId="6" priority="1" operator="beginsWith" text="Ok">
       <formula>LEFT(N33,2)="Ok"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N33 N42 N45 N79 N84 N95 N114 N116 N123 N136 N137 N138 N11 N13 N14 N15 N16 N17 N18 S2 S3 S4 S5">
+  <conditionalFormatting sqref="N33 N42 N45 N79 N84 N95 N114 N117 N124 N137 N138 N139 N11 N13 N14 N15 N16 N17 N18 S2 S3 S4 S5">
     <cfRule type="beginsWith" dxfId="5" priority="2" operator="beginsWith" text="Não se aplica">
       <formula>LEFT(N33,13)="Não se aplica"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Dimensionamento pilar: estribos escalonados por zonas conforme o cortante ao longo da altura; taxa de estribos pelas zonas; dados da versão do usuário
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01STLw65tKW2EfXfQSwTwwMc
</commit_message>
<xml_diff>
--- a/3 - EMPUXO DE MUROS DE ARRIMO.xlsx
+++ b/3 - EMPUXO DE MUROS DE ARRIMO.xlsx
@@ -25,7 +25,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'CONTENÇÃO RÁPIDA'!$K$1:$T$259</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'DIMENSIONAMENTO PILAR'!$K$1:$T$147</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'DIMENSIONAMENTO PILAR'!$K$1:$T$165</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1" iterateCount="1000"/>
   <extLst>
@@ -2689,7 +2689,7 @@
                   <c:v>0.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2723,10 +2723,10 @@
                   <c:v>0.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>17.247957670388743</c:v>
+                  <c:v>12.167266237259694</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>172.47957670388743</c:v>
+                  <c:v>187.3759000537993</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0.0</c:v>
@@ -2741,10 +2741,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0.0</c:v>
@@ -2782,10 +2782,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>17.247957670388743</c:v>
+                  <c:v>12.167266237259694</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>17.247957670388743</c:v>
+                  <c:v>12.167266237259694</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2797,7 +2797,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.0</c:v>
@@ -2832,7 +2832,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>146.60764019830432</c:v>
+                  <c:v>158.17446108437605</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.0</c:v>
@@ -2847,10 +2847,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0.4166666666666667</c:v>
+                  <c:v>0.6666666666666666</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.4166666666666667</c:v>
+                  <c:v>0.6666666666666666</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2882,7 +2882,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>120.73570369272119</c:v>
+                  <c:v>128.97302211495278</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.0</c:v>
@@ -2897,10 +2897,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0.8333333333333334</c:v>
+                  <c:v>1.3333333333333333</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.8333333333333334</c:v>
+                  <c:v>1.3333333333333333</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2932,7 +2932,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>94.86376718713808</c:v>
+                  <c:v>99.7715831455295</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.0</c:v>
@@ -2947,10 +2947,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>1.25</c:v>
+                  <c:v>2.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.25</c:v>
+                  <c:v>2.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2982,7 +2982,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>68.99183068155496</c:v>
+                  <c:v>70.57014417610624</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.0</c:v>
@@ -2997,10 +2997,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>1.6666666666666667</c:v>
+                  <c:v>2.6666666666666665</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.6666666666666667</c:v>
+                  <c:v>2.6666666666666665</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3032,7 +3032,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>43.119894175971865</c:v>
+                  <c:v>41.36870520668296</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.0</c:v>
@@ -3047,10 +3047,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>2.0833333333333335</c:v>
+                  <c:v>3.3333333333333335</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.0833333333333335</c:v>
+                  <c:v>3.3333333333333335</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3082,7 +3082,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>198.35151320947054</c:v>
+                  <c:v>215.4822850618692</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.0</c:v>
@@ -3097,10 +3097,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0.9090909090909092</c:v>
+                  <c:v>1.4146341463414631</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.9090909090909092</c:v>
+                  <c:v>1.4146341463414631</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3135,7 +3135,7 @@
                   <c:v>0.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-60.367851846360594</c:v>
+                  <c:v>-65.58156501882975</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3147,10 +3147,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3185,7 +3185,7 @@
                   <c:v>0.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-60.367851846360594</c:v>
+                  <c:v>-65.58156501882975</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3216,7 +3216,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>p,topo = 17,25 kN/m</c:v>
+                  <c:v>p,topo = 12,17 kN/m</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3260,7 +3260,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>17.247957670388743</c:v>
+                  <c:v>12.167266237259694</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3272,7 +3272,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3288,7 +3288,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>p,base = 172,48 kN/m</c:v>
+                  <c:v>p,base = 187,38 kN/m</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3332,7 +3332,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>172.47957670388743</c:v>
+                  <c:v>187.3759000537993</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3360,7 +3360,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>E = 237,2 kN (y = 0,91 m)</c:v>
+                  <c:v>E = 399,1 kN (y = 1,41 m)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3404,7 +3404,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>198.35151320947054</c:v>
+                  <c:v>215.4822850618692</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3416,7 +3416,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0.9090909090909092</c:v>
+                  <c:v>1.4146341463414631</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3432,7 +3432,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>R,topo = 55,0 kN → laje</c:v>
+                  <c:v>R,topo = 88,3 kN → laje</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3476,7 +3476,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>-60.367851846360594</c:v>
+                  <c:v>-65.58156501882975</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3488,7 +3488,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3504,7 +3504,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>R,base = 182,2 kN</c:v>
+                  <c:v>R,base = 310,8 kN</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3548,7 +3548,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>-60.367851846360594</c:v>
+                  <c:v>-65.58156501882975</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3793,7 +3793,7 @@
                   <c:v>0.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3830,7 +3830,7 @@
                   <c:v>2.639320225002103</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>26.39320225002103</c:v>
+                  <c:v>40.645531465032384</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0.0</c:v>
@@ -3845,10 +3845,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0.0</c:v>
@@ -3901,7 +3901,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.0</c:v>
@@ -3936,7 +3936,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>20.4547317437663</c:v>
+                  <c:v>31.143978655024814</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.0</c:v>
@@ -3951,10 +3951,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0.625</c:v>
+                  <c:v>1.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.625</c:v>
+                  <c:v>1.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3986,7 +3986,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>14.516261237511566</c:v>
+                  <c:v>21.642425845017243</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.0</c:v>
@@ -4001,10 +4001,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>1.25</c:v>
+                  <c:v>2.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.25</c:v>
+                  <c:v>2.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4036,7 +4036,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>8.577790731256833</c:v>
+                  <c:v>12.140873035009673</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.0</c:v>
@@ -4051,10 +4051,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>1.875</c:v>
+                  <c:v>3.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.875</c:v>
+                  <c:v>3.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4085,64 +4085,64 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
                 <c:pt idx="0">
-                  <c:v>26.393202250021027</c:v>
+                  <c:v>40.645531465032384</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>26.393202250021027</c:v>
+                  <c:v>40.645531465032384</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>28.768590452522922</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>28.768590452522922</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>16.89164944001346</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>16.89164944001346</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>5.0147084275039955</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>5.0147084275039955</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>5.0147084275039955</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>5.0147084275039955</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>5.0147084275039955</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>5.0147084275039955</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>5.0147084275039955</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>5.0147084275039955</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>5.0147084275039955</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>5.0147084275039955</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>5.0147084275039955</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>5.0147084275039955</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>5.0147084275039955</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>5.0147084275039955</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4169,49 +4169,49 @@
                   <c:v>2.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2.5</c:v>
+                  <c:v>3.75</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2.5</c:v>
+                  <c:v>3.75</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4246,7 +4246,7 @@
                   <c:v>0.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>27.71286236252208</c:v>
+                  <c:v>42.677808038284006</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4292,6 +4292,12 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>42.677808038284006</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -4336,6 +4342,12 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>42.677808038284006</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -4685,7 +4697,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>2.5</c:v>
+                  <c:v>4.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4701,7 +4713,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>σ,base = 26,39 kN/m² = solo 23,75 + Sc 2,64</c:v>
+                  <c:v>σ,base = 40,65 kN/m² = solo 38,01 + Sc 2,64</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -4745,7 +4757,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>26.39320225002103</c:v>
+                  <c:v>40.645531465032384</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4773,7 +4785,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>P1: g = 29,69 | q = 3,30 kN/m</c:v>
+                  <c:v>P1: g = 47,51 | q = 3,30 kN/m</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -4817,7 +4829,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>26.393202250021027</c:v>
+                  <c:v>40.645531465032384</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4845,7 +4857,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>P2: g = 14,85 | q = 3,30 kN/m</c:v>
+                  <c:v>P2: g = 32,66 | q = 3,30 kN/m</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -4889,7 +4901,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>14.516261237511564</c:v>
+                  <c:v>28.768590452522922</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4917,7 +4929,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v/>
+                  <c:v>P3: g = 17,82 | q = 3,30 kN/m</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -4960,6 +4972,9 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>16.89164944001346</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -4969,6 +4984,9 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>3.125</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -4983,7 +5001,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v/>
+                  <c:v>P4: g = 0,59 | q = 0,66 kN/m</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5026,6 +5044,9 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>5.0147084275039955</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -5035,6 +5056,9 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>3.875</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -13651,7 +13675,7 @@
         </is>
       </c>
       <c r="L33" s="224">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="M33" s="231" t="inlineStr">
         <is>
@@ -13671,7 +13695,7 @@
         </is>
       </c>
       <c r="L34" s="226">
-        <f>13.07/2</f>
+        <f>9.22/2</f>
       </c>
       <c r="M34" s="231" t="inlineStr">
         <is>
@@ -16543,7 +16567,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="K1:T147"/>
+  <dimension ref="K1:T165"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="10" max="10" width="2.7109375" customWidth="1"/>
@@ -16582,7 +16606,7 @@
       </c>
       <c r="N2" s="240"/>
       <c r="O2" s="241">
-        <v>12.5</v>
+        <v>20</v>
       </c>
       <c r="P2" s="240">
         <f>$L$111&amp;" barras em cada face ("&amp;FIXED($L$112,2)&amp;" cm²) | espaço livre "&amp;FIXED($L$117,2)&amp;" cm"</f>
@@ -16602,19 +16626,19 @@
       </c>
       <c r="L3" s="239"/>
       <c r="M3" s="240">
-        <f>"Asw,nec = "&amp;FIXED($L$133,2)&amp;" cm²/m"</f>
+        <f>"Asw,nec = "&amp;FIXED($L$133,2)&amp;" cm²/m (máx.)"</f>
       </c>
       <c r="N3" s="240"/>
       <c r="O3" s="241">
         <v>6.3</v>
       </c>
       <c r="P3" s="240">
-        <f>"c/ "&amp;$L$137&amp;" cm ("&amp;$L$43&amp;" ramos) = "&amp;FIXED($L$138,2)&amp;" cm²/m"</f>
+        <f>("Ø"&amp;$L$41&amp;": "&amp;IF(N148&lt;=0,"","c/"&amp;S148&amp;" ("&amp;FIXED(L148,1)&amp;"–"&amp;FIXED(M148,1)&amp;" m)")&amp;IF(N149&lt;=0,""," | "&amp;"c/"&amp;S149&amp;" ("&amp;FIXED(L149,1)&amp;"–"&amp;FIXED(M149,1)&amp;" m)")&amp;IF(N150&lt;=0,""," | "&amp;"c/"&amp;S150&amp;" ("&amp;FIXED(L150,1)&amp;"–"&amp;FIXED(M150,1)&amp;" m)")&amp;IF(N151&lt;=0,""," | "&amp;"c/"&amp;S151&amp;" ("&amp;FIXED(L151,1)&amp;"–"&amp;FIXED(M151,1)&amp;" m)")&amp;IF(N152&lt;=0,""," | "&amp;"c/"&amp;S152&amp;" ("&amp;FIXED(L152,1)&amp;"–"&amp;FIXED(M152,1)&amp;" m)")&amp;IF(N153&lt;=0,""," | "&amp;"c/"&amp;S153&amp;" ("&amp;FIXED(L153,1)&amp;"–"&amp;FIXED(M153,1)&amp;" m)"))</f>
       </c>
       <c r="Q3" s="240"/>
       <c r="R3" s="240"/>
       <c r="S3" s="242">
-        <f>IF($L$123&gt;$L$124,"NÃO OK – biela: aumentar seção",IF($L$137&lt;5,"NÃO OK – s &lt; 5 cm: aumentar Ø",IF($L$41&lt;$L$139,"NÃO OK – Ø,t &lt; Ø,l/4","OK")))</f>
+        <f>IF($L$123&gt;$L$124,"NÃO OK – biela: aumentar seção",IF($L$41&lt;$L$139,"NÃO OK – Ø,t &lt; Ø,l/4",(IF(ABS($L$155-$L$142)&gt;0.01,"NÃO OK – soma das zonas ≠ H",IF($L$156&lt;5,"NÃO OK – s &lt; 5 cm: aumentar Ø","OK")))))</f>
       </c>
       <c r="T3" s="242"/>
     </row>
@@ -16652,7 +16676,7 @@
       </c>
       <c r="N5" s="240"/>
       <c r="O5" s="240">
-        <f>"Longit. "&amp;FIXED($L$144,1)&amp;" + estribos "&amp;FIXED($L$146,1)&amp;" = "&amp;FIXED($L$147,1)&amp;" kg/m³"</f>
+        <f>"Longit. "&amp;FIXED($L$161,1)&amp;" + estribos "&amp;FIXED($L$163,1)&amp;" = "&amp;FIXED($L$165,1)&amp;" kg/m³"</f>
       </c>
       <c r="P5" s="240"/>
       <c r="Q5" s="240"/>
@@ -16861,11 +16885,11 @@
         </is>
       </c>
       <c r="L18" s="236">
-        <f>"Ø"&amp;$L$41&amp;" c/"&amp;$L$137&amp;" ("&amp;$L$43&amp;" ramos)"</f>
+        <f>"Ø"&amp;$L$41&amp;" – "&amp;$L$154&amp;" estribos"</f>
       </c>
       <c r="M18" s="236"/>
       <c r="N18" s="232">
-        <f>IF($L$137&lt;5,"s &lt; 5 cm – aumentar Ø,t",IF($L$138&gt;=$L$133,"Ok","Rever"))</f>
+        <f>(IF(ABS($L$155-$L$142)&gt;0.01,"NÃO OK – soma das zonas ≠ H",IF($L$156&lt;5,"NÃO OK – s &lt; 5 cm: aumentar Ø","OK")))</f>
       </c>
       <c r="O18" s="233" t="inlineStr">
         <is>
@@ -16923,7 +16947,7 @@
         </is>
       </c>
       <c r="L30" s="224">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="M30" s="231" t="inlineStr">
         <is>
@@ -16943,7 +16967,7 @@
         </is>
       </c>
       <c r="L31" s="224">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="M31" s="231" t="inlineStr">
         <is>
@@ -16970,7 +16994,7 @@
         </is>
       </c>
       <c r="L33" s="224">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="M33" s="231" t="inlineStr">
         <is>
@@ -17060,7 +17084,7 @@
         </is>
       </c>
       <c r="L38" s="224">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="M38" s="231" t="inlineStr">
         <is>
@@ -17080,7 +17104,7 @@
         </is>
       </c>
       <c r="L39" s="224">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="M39" s="231" t="inlineStr">
         <is>
@@ -18561,7 +18585,7 @@
     <row r="137">
       <c r="K137" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">s</t>
+          <t xml:space="preserve">s,unif</t>
         </is>
       </c>
       <c r="L137" s="229">
@@ -18577,7 +18601,7 @@
       </c>
       <c r="O137" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Espaçamento adotado (arredondado para baixo).</t>
+          <t xml:space="preserve">Espaçamento se usar o Vsd máximo em toda a altura (sem escalonamento).</t>
         </is>
       </c>
     </row>
@@ -18627,124 +18651,577 @@
         </is>
       </c>
     </row>
-    <row r="141">
-      <c r="K141" s="221" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7 . TAXA DE AÇO</t>
-        </is>
-      </c>
-      <c r="L141" s="221"/>
-      <c r="M141" s="221"/>
-      <c r="N141" s="221"/>
-      <c r="O141" s="221"/>
-      <c r="P141" s="221"/>
-      <c r="Q141" s="221"/>
-      <c r="R141" s="221"/>
-      <c r="S141" s="221"/>
-      <c r="T141" s="221"/>
+    <row r="140">
+      <c r="K140" s="222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.3 Estribos por zonas (escalonamento ao longo da altura)</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="32" customHeight="1">
+      <c r="K141" s="220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O cortante cai da base para o topo, então cada zona usa o maior |V| do seu trecho (e não o Vsd máximo em toda a altura). V(z) = R,base − p,base·z + Δp·z²/(2H), com z medido da base. Os comprimentos das zonas são cinza: pode editar.</t>
+        </is>
+      </c>
+      <c r="L141" s="220"/>
+      <c r="M141" s="220"/>
+      <c r="N141" s="220"/>
+      <c r="O141" s="220"/>
+      <c r="P141" s="220"/>
+      <c r="Q141" s="220"/>
+      <c r="R141" s="220"/>
+      <c r="S141" s="220"/>
+      <c r="T141" s="220"/>
+    </row>
+    <row r="142">
+      <c r="K142" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H</t>
+        </is>
+      </c>
+      <c r="L142" s="227">
+        <f>'CONTENÇÃO RÁPIDA'!$L$33</f>
+      </c>
+      <c r="M142" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">m</t>
+        </is>
+      </c>
+      <c r="O142" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Altura do pilar carregada (aba CONTENÇÃO RÁPIDA).</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="K143" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">ρ,aço</t>
-        </is>
-      </c>
-      <c r="L143" s="224">
-        <v>0.785</v>
+          <t xml:space="preserve">p,base</t>
+        </is>
+      </c>
+      <c r="L143" s="227">
+        <f>'CONTENÇÃO RÁPIDA'!$L$60</f>
       </c>
       <c r="M143" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">kg/m/cm²</t>
+          <t xml:space="preserve">kN/m</t>
         </is>
       </c>
       <c r="O143" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peso por metro de 1 cm² de barra (7850 kg/m³).</t>
+          <t xml:space="preserve">Carga na base (aba CONTENÇÃO RÁPIDA).</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="K144" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Longit.</t>
+          <t xml:space="preserve">Δp</t>
         </is>
       </c>
       <c r="L144" s="227">
-        <f>$L$113*$L$143/($L$39*$L$38/10000)</f>
+        <f>'CONTENÇÃO RÁPIDA'!$L$61</f>
       </c>
       <c r="M144" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">kg/m³</t>
+          <t xml:space="preserve">kN/m</t>
         </is>
       </c>
       <c r="O144" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Armadura longitudinal (duas faces) por m³ de concreto.</t>
+          <t xml:space="preserve">Parcela triangular (aba CONTENÇÃO RÁPIDA).</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="K145" s="223" t="inlineStr">
         <is>
-          <t xml:space="preserve">l,est</t>
+          <t xml:space="preserve">R,base</t>
         </is>
       </c>
       <c r="L145" s="227">
-        <f>2*($L$39+$L$38)-8*$L$40+12</f>
+        <f>IFERROR(INDEX('CONTENÇÃO RÁPIDA'!$M$74:$M$76,MATCH($L$45,'CONTENÇÃO RÁPIDA'!$K$74:$K$76,0)),0)</f>
       </c>
       <c r="M145" s="231" t="inlineStr">
         <is>
-          <t xml:space="preserve">cm</t>
+          <t xml:space="preserve">kN</t>
         </is>
       </c>
       <c r="O145" s="233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comprimento de cada estribo (perímetro − cobrimentos + ganchos).</t>
+          <t xml:space="preserve">Reação na base do modelo escolhido.</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="K146" s="223" t="inlineStr">
         <is>
+          <t xml:space="preserve">zonas</t>
+        </is>
+      </c>
+      <c r="L146" s="224">
+        <v>3</v>
+      </c>
+      <c r="M146" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">un</t>
+        </is>
+      </c>
+      <c r="N146" s="232">
+        <f>IF(OR($L$146&lt;1,$L$146&gt;6),"Rever: 1 a 6 zonas","Ok")</f>
+      </c>
+      <c r="O146" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Número de zonas de mesmo comprimento (1 a 6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="30" customHeight="1">
+      <c r="K147" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zona</t>
+        </is>
+      </c>
+      <c r="L147" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">z,início (m)</t>
+        </is>
+      </c>
+      <c r="M147" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">z,fim (m)</t>
+        </is>
+      </c>
+      <c r="N147" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compr. (m)</t>
+        </is>
+      </c>
+      <c r="O147" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vk,máx (kN)</t>
+        </is>
+      </c>
+      <c r="P147" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vsd (kN)</t>
+        </is>
+      </c>
+      <c r="Q147" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asw (cm²/m)</t>
+        </is>
+      </c>
+      <c r="R147" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s,calc (cm)</t>
+        </is>
+      </c>
+      <c r="S147" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s (cm)</t>
+        </is>
+      </c>
+      <c r="T147" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nº estribos</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="K148" s="237">
+        <v>1</v>
+      </c>
+      <c r="L148" s="227">
+        <v>0</v>
+      </c>
+      <c r="M148" s="227">
+        <f>L148+N148</f>
+      </c>
+      <c r="N148" s="225">
+        <f>IF(1&lt;=$L$146,$L$142/$L$146,0)</f>
+      </c>
+      <c r="O148" s="227">
+        <f>IF(N148&lt;=0,"",MAX(ABS(($L$145-$L$143*L148+$L$144*L148^2/(2*$L$142))),ABS(($L$145-$L$143*M148+$L$144*M148^2/(2*$L$142)))))</f>
+      </c>
+      <c r="P148" s="227">
+        <f>IF(N148&lt;=0,"",O148*$L$29)</f>
+      </c>
+      <c r="Q148" s="227">
+        <f>IF(N148&lt;=0,"",MAX(MAX(0,P148-$L$127)/(0.9*$L$76*$L$129/10)*100,$L$132))</f>
+      </c>
+      <c r="R148" s="227">
+        <f>IF(N148&lt;=0,"",$L$43*PI()*($L$41/10)^2/4/Q148*100)</f>
+      </c>
+      <c r="S148" s="229">
+        <f>IF(N148&lt;=0,"",ROUNDDOWN(MIN(R148,IF(P148&lt;=0.67*$L$124,MIN(0.6*$L$76,30),MIN(0.3*$L$76,20)),$L$136),0))</f>
+      </c>
+      <c r="T148" s="229">
+        <f>IF(N148&lt;=0,"",ROUNDUP(N148*100/S148,0))</f>
+      </c>
+    </row>
+    <row r="149">
+      <c r="K149" s="237">
+        <v>2</v>
+      </c>
+      <c r="L149" s="227">
+        <f>M148</f>
+      </c>
+      <c r="M149" s="227">
+        <f>L149+N149</f>
+      </c>
+      <c r="N149" s="225">
+        <f>IF(2&lt;=$L$146,$L$142/$L$146,0)</f>
+      </c>
+      <c r="O149" s="227">
+        <f>IF(N149&lt;=0,"",MAX(ABS(($L$145-$L$143*L149+$L$144*L149^2/(2*$L$142))),ABS(($L$145-$L$143*M149+$L$144*M149^2/(2*$L$142)))))</f>
+      </c>
+      <c r="P149" s="227">
+        <f>IF(N149&lt;=0,"",O149*$L$29)</f>
+      </c>
+      <c r="Q149" s="227">
+        <f>IF(N149&lt;=0,"",MAX(MAX(0,P149-$L$127)/(0.9*$L$76*$L$129/10)*100,$L$132))</f>
+      </c>
+      <c r="R149" s="227">
+        <f>IF(N149&lt;=0,"",$L$43*PI()*($L$41/10)^2/4/Q149*100)</f>
+      </c>
+      <c r="S149" s="229">
+        <f>IF(N149&lt;=0,"",ROUNDDOWN(MIN(R149,IF(P149&lt;=0.67*$L$124,MIN(0.6*$L$76,30),MIN(0.3*$L$76,20)),$L$136),0))</f>
+      </c>
+      <c r="T149" s="229">
+        <f>IF(N149&lt;=0,"",ROUNDUP(N149*100/S149,0))</f>
+      </c>
+    </row>
+    <row r="150">
+      <c r="K150" s="237">
+        <v>3</v>
+      </c>
+      <c r="L150" s="227">
+        <f>M149</f>
+      </c>
+      <c r="M150" s="227">
+        <f>L150+N150</f>
+      </c>
+      <c r="N150" s="225">
+        <f>IF(3&lt;=$L$146,$L$142/$L$146,0)</f>
+      </c>
+      <c r="O150" s="227">
+        <f>IF(N150&lt;=0,"",MAX(ABS(($L$145-$L$143*L150+$L$144*L150^2/(2*$L$142))),ABS(($L$145-$L$143*M150+$L$144*M150^2/(2*$L$142)))))</f>
+      </c>
+      <c r="P150" s="227">
+        <f>IF(N150&lt;=0,"",O150*$L$29)</f>
+      </c>
+      <c r="Q150" s="227">
+        <f>IF(N150&lt;=0,"",MAX(MAX(0,P150-$L$127)/(0.9*$L$76*$L$129/10)*100,$L$132))</f>
+      </c>
+      <c r="R150" s="227">
+        <f>IF(N150&lt;=0,"",$L$43*PI()*($L$41/10)^2/4/Q150*100)</f>
+      </c>
+      <c r="S150" s="229">
+        <f>IF(N150&lt;=0,"",ROUNDDOWN(MIN(R150,IF(P150&lt;=0.67*$L$124,MIN(0.6*$L$76,30),MIN(0.3*$L$76,20)),$L$136),0))</f>
+      </c>
+      <c r="T150" s="229">
+        <f>IF(N150&lt;=0,"",ROUNDUP(N150*100/S150,0))</f>
+      </c>
+    </row>
+    <row r="151">
+      <c r="K151" s="237">
+        <v>4</v>
+      </c>
+      <c r="L151" s="227">
+        <f>M150</f>
+      </c>
+      <c r="M151" s="227">
+        <f>L151+N151</f>
+      </c>
+      <c r="N151" s="225">
+        <f>IF(4&lt;=$L$146,$L$142/$L$146,0)</f>
+      </c>
+      <c r="O151" s="227">
+        <f>IF(N151&lt;=0,"",MAX(ABS(($L$145-$L$143*L151+$L$144*L151^2/(2*$L$142))),ABS(($L$145-$L$143*M151+$L$144*M151^2/(2*$L$142)))))</f>
+      </c>
+      <c r="P151" s="227">
+        <f>IF(N151&lt;=0,"",O151*$L$29)</f>
+      </c>
+      <c r="Q151" s="227">
+        <f>IF(N151&lt;=0,"",MAX(MAX(0,P151-$L$127)/(0.9*$L$76*$L$129/10)*100,$L$132))</f>
+      </c>
+      <c r="R151" s="227">
+        <f>IF(N151&lt;=0,"",$L$43*PI()*($L$41/10)^2/4/Q151*100)</f>
+      </c>
+      <c r="S151" s="229">
+        <f>IF(N151&lt;=0,"",ROUNDDOWN(MIN(R151,IF(P151&lt;=0.67*$L$124,MIN(0.6*$L$76,30),MIN(0.3*$L$76,20)),$L$136),0))</f>
+      </c>
+      <c r="T151" s="229">
+        <f>IF(N151&lt;=0,"",ROUNDUP(N151*100/S151,0))</f>
+      </c>
+    </row>
+    <row r="152">
+      <c r="K152" s="237">
+        <v>5</v>
+      </c>
+      <c r="L152" s="227">
+        <f>M151</f>
+      </c>
+      <c r="M152" s="227">
+        <f>L152+N152</f>
+      </c>
+      <c r="N152" s="225">
+        <f>IF(5&lt;=$L$146,$L$142/$L$146,0)</f>
+      </c>
+      <c r="O152" s="227">
+        <f>IF(N152&lt;=0,"",MAX(ABS(($L$145-$L$143*L152+$L$144*L152^2/(2*$L$142))),ABS(($L$145-$L$143*M152+$L$144*M152^2/(2*$L$142)))))</f>
+      </c>
+      <c r="P152" s="227">
+        <f>IF(N152&lt;=0,"",O152*$L$29)</f>
+      </c>
+      <c r="Q152" s="227">
+        <f>IF(N152&lt;=0,"",MAX(MAX(0,P152-$L$127)/(0.9*$L$76*$L$129/10)*100,$L$132))</f>
+      </c>
+      <c r="R152" s="227">
+        <f>IF(N152&lt;=0,"",$L$43*PI()*($L$41/10)^2/4/Q152*100)</f>
+      </c>
+      <c r="S152" s="229">
+        <f>IF(N152&lt;=0,"",ROUNDDOWN(MIN(R152,IF(P152&lt;=0.67*$L$124,MIN(0.6*$L$76,30),MIN(0.3*$L$76,20)),$L$136),0))</f>
+      </c>
+      <c r="T152" s="229">
+        <f>IF(N152&lt;=0,"",ROUNDUP(N152*100/S152,0))</f>
+      </c>
+    </row>
+    <row r="153">
+      <c r="K153" s="237">
+        <v>6</v>
+      </c>
+      <c r="L153" s="227">
+        <f>M152</f>
+      </c>
+      <c r="M153" s="227">
+        <f>L153+N153</f>
+      </c>
+      <c r="N153" s="225">
+        <f>IF(6&lt;=$L$146,$L$142/$L$146,0)</f>
+      </c>
+      <c r="O153" s="227">
+        <f>IF(N153&lt;=0,"",MAX(ABS(($L$145-$L$143*L153+$L$144*L153^2/(2*$L$142))),ABS(($L$145-$L$143*M153+$L$144*M153^2/(2*$L$142)))))</f>
+      </c>
+      <c r="P153" s="227">
+        <f>IF(N153&lt;=0,"",O153*$L$29)</f>
+      </c>
+      <c r="Q153" s="227">
+        <f>IF(N153&lt;=0,"",MAX(MAX(0,P153-$L$127)/(0.9*$L$76*$L$129/10)*100,$L$132))</f>
+      </c>
+      <c r="R153" s="227">
+        <f>IF(N153&lt;=0,"",$L$43*PI()*($L$41/10)^2/4/Q153*100)</f>
+      </c>
+      <c r="S153" s="229">
+        <f>IF(N153&lt;=0,"",ROUNDDOWN(MIN(R153,IF(P153&lt;=0.67*$L$124,MIN(0.6*$L$76,30),MIN(0.3*$L$76,20)),$L$136),0))</f>
+      </c>
+      <c r="T153" s="229">
+        <f>IF(N153&lt;=0,"",ROUNDUP(N153*100/S153,0))</f>
+      </c>
+    </row>
+    <row r="154">
+      <c r="K154" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
+      </c>
+      <c r="L154" s="229">
+        <f>SUM(T148:T153)</f>
+      </c>
+      <c r="M154" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">estr.</t>
+        </is>
+      </c>
+      <c r="O154" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Número total de estribos no pilar (escalonados).</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="K155" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ΣL</t>
+        </is>
+      </c>
+      <c r="L155" s="227">
+        <f>SUM(N148:N153)</f>
+      </c>
+      <c r="M155" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">m</t>
+        </is>
+      </c>
+      <c r="N155" s="232">
+        <f>IF(ABS($L$155-$L$142)&gt;0.01,"Rever: soma ≠ H","Ok")</f>
+      </c>
+      <c r="O155" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Soma dos comprimentos das zonas (deve ser igual a H).</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="K156" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s,mín</t>
+        </is>
+      </c>
+      <c r="L156" s="229">
+        <f>MIN(S148:S153)</f>
+      </c>
+      <c r="M156" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O156" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Menor espaçamento entre as zonas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="K158" s="221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7 . TAXA DE AÇO</t>
+        </is>
+      </c>
+      <c r="L158" s="221"/>
+      <c r="M158" s="221"/>
+      <c r="N158" s="221"/>
+      <c r="O158" s="221"/>
+      <c r="P158" s="221"/>
+      <c r="Q158" s="221"/>
+      <c r="R158" s="221"/>
+      <c r="S158" s="221"/>
+      <c r="T158" s="221"/>
+    </row>
+    <row r="160">
+      <c r="K160" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ρ,aço</t>
+        </is>
+      </c>
+      <c r="L160" s="224">
+        <v>0.785</v>
+      </c>
+      <c r="M160" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kg/m/cm²</t>
+        </is>
+      </c>
+      <c r="O160" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peso por metro de 1 cm² de barra (7850 kg/m³).</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="K161" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Longit.</t>
+        </is>
+      </c>
+      <c r="L161" s="227">
+        <f>$L$113*$L$160/($L$39*$L$38/10000)</f>
+      </c>
+      <c r="M161" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kg/m³</t>
+        </is>
+      </c>
+      <c r="O161" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Armadura longitudinal (duas faces) por m³ de concreto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="K162" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">l,est</t>
+        </is>
+      </c>
+      <c r="L162" s="227">
+        <f>2*($L$39+$L$38)-8*$L$40+12</f>
+      </c>
+      <c r="M162" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
+      <c r="O162" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comprimento de cada estribo (perímetro − cobrimentos + ganchos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="K163" s="223" t="inlineStr">
+        <is>
           <t xml:space="preserve">Estribos</t>
         </is>
       </c>
-      <c r="L146" s="227">
-        <f>100/$L$137*$L$145/100*PI()*($L$41/10)^2/4*$L$143*$L$43/2/($L$39*$L$38/10000)</f>
-      </c>
-      <c r="M146" s="231" t="inlineStr">
+      <c r="L163" s="227">
+        <f>$L$154*$L$162/100*PI()*($L$41/10)^2/4*$L$160*$L$43/2/($L$39*$L$38/10000*$L$142)</f>
+      </c>
+      <c r="M163" s="231" t="inlineStr">
         <is>
           <t xml:space="preserve">kg/m³</t>
         </is>
       </c>
-      <c r="O146" s="233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estribos por m³ de concreto (100/s estribos por metro).</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="K147" s="223" t="inlineStr">
+      <c r="O163" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estribos escalonados (item 6.3) por m³ de concreto do pilar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="K164" s="223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estr. unif.</t>
+        </is>
+      </c>
+      <c r="L164" s="227">
+        <f>100/$L$137*$L$162/100*PI()*($L$41/10)^2/4*$L$160*$L$43/2/($L$39*$L$38/10000)</f>
+      </c>
+      <c r="M164" s="231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kg/m³</t>
+        </is>
+      </c>
+      <c r="O164" s="233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comparação: estribos com s,unif em toda a altura.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="K165" s="223" t="inlineStr">
         <is>
           <t xml:space="preserve">Total</t>
         </is>
       </c>
-      <c r="L147" s="227">
-        <f>$L$144+$L$146</f>
-      </c>
-      <c r="M147" s="231" t="inlineStr">
+      <c r="L165" s="227">
+        <f>$L$161+$L$163</f>
+      </c>
+      <c r="M165" s="231" t="inlineStr">
         <is>
           <t xml:space="preserve">kg/m³</t>
         </is>
       </c>
-      <c r="O147" s="233" t="inlineStr">
+      <c r="O165" s="233" t="inlineStr">
         <is>
           <t xml:space="preserve">Taxa total de aço do pilar.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="39">
     <mergeCell ref="K1:T1"/>
     <mergeCell ref="K6:T6"/>
     <mergeCell ref="K8:T8"/>
@@ -18757,6 +19234,7 @@
     <mergeCell ref="K119:T119"/>
     <mergeCell ref="K121:T121"/>
     <mergeCell ref="K141:T141"/>
+    <mergeCell ref="K158:T158"/>
     <mergeCell ref="L10:M10"/>
     <mergeCell ref="O10:T10"/>
     <mergeCell ref="L11:M11"/>
@@ -18784,12 +19262,12 @@
     <mergeCell ref="O5:R5"/>
     <mergeCell ref="S5:T5"/>
   </mergeCells>
-  <conditionalFormatting sqref="N33 N42 N45 N79 N84 N95 N114 N117 N124 N137 N138 N139 N11 N13 N14 N15 N16 N17 N18 S2 S3 S4 S5">
+  <conditionalFormatting sqref="N33 N42 N45 N79 N84 N95 N114 N117 N124 N137 N138 N139 N146 N155 N11 N13 N14 N15 N16 N17 N18 S2 S3 S4 S5">
     <cfRule type="beginsWith" dxfId="6" priority="1" operator="beginsWith" text="Ok">
       <formula>LEFT(N33,2)="Ok"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N33 N42 N45 N79 N84 N95 N114 N117 N124 N137 N138 N139 N11 N13 N14 N15 N16 N17 N18 S2 S3 S4 S5">
+  <conditionalFormatting sqref="N33 N42 N45 N79 N84 N95 N114 N117 N124 N137 N138 N139 N146 N155 N11 N13 N14 N15 N16 N17 N18 S2 S3 S4 S5">
     <cfRule type="beginsWith" dxfId="5" priority="2" operator="beginsWith" text="Não se aplica">
       <formula>LEFT(N33,13)="Não se aplica"</formula>
     </cfRule>

</xml_diff>